<commit_message>
Realinha fase de persona com o padrao real de producao do CDRVIEW
Persona (K-Means+XGBoost) passa da Fase 5 para a Fase 1: retreino
trimestral batch + scoring semanal/incremental sao dois jobs agendados
sobre o tensor do CDRVIEW, sem exigir a infraestrutura de streaming por
evento que Markov/IPED/Vamping (rede e engajamento) de fato precisam.
Atualiza planilha (sprints, alocacao, custo) e PDF de arquitetura.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/JOURNEYGRAPH_MNO_PLANO_IMPLEMENTACAO_CLARO.xlsx
+++ b/docs/JOURNEYGRAPH_MNO_PLANO_IMPLEMENTACAO_CLARO.xlsx
@@ -102,11 +102,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FBE6E6"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="002E8B62"/>
       </patternFill>
     </fill>
@@ -128,6 +123,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="003A7CA5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FBE6E6"/>
       </patternFill>
     </fill>
   </fills>
@@ -157,7 +157,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -184,9 +184,6 @@
     </xf>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -218,11 +215,11 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="11" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="12" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="13" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="9" fontId="3" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -233,7 +230,7 @@
     <xf numFmtId="9" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="3" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="9" fontId="3" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -601,7 +598,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H18"/>
+  <dimension ref="A1:H19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -688,14 +685,14 @@
       </c>
       <c r="C5" s="7" t="inlineStr">
         <is>
-          <t>Segmentação real (K-Means+XGBoost), IPED e Vamping para Marketing/CRM, 1 região piloto, sobre tensor longitudinal que a GUI Análises do CDRVIEW já sabe exportar.</t>
+          <t>Segmentação real (K-Means+XGBoost), IPED e Vamping para Marketing/CRM, 1 região piloto, sobre tensor longitudinal que a GUI Análises do CDRVIEW já sabe exportar. Persona já sai no padrão real de produção da Claro: retreino K-Means trimestral batch + scoring XGBoost semanal/incremental — dois jobs agendados sobre o tensor, sem infraestrutura de streaming nova.</t>
         </is>
       </c>
       <c r="D5" s="7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E5" s="7" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F5" s="8" t="inlineStr">
         <is>
@@ -708,7 +705,7 @@
         </is>
       </c>
       <c r="H5" s="10">
-        <f>'Custo Detalhado'!G12</f>
+        <f>'Custo Detalhado'!G13</f>
         <v/>
       </c>
     </row>
@@ -743,7 +740,7 @@
         </is>
       </c>
       <c r="H6" s="10">
-        <f>'Custo Detalhado'!G18</f>
+        <f>'Custo Detalhado'!G19</f>
         <v/>
       </c>
     </row>
@@ -778,7 +775,7 @@
         </is>
       </c>
       <c r="H7" s="10">
-        <f>'Custo Detalhado'!G26</f>
+        <f>'Custo Detalhado'!G27</f>
         <v/>
       </c>
     </row>
@@ -813,7 +810,7 @@
         </is>
       </c>
       <c r="H8" s="10">
-        <f>'Custo Detalhado'!G36</f>
+        <f>'Custo Detalhado'!G37</f>
         <v/>
       </c>
     </row>
@@ -823,32 +820,32 @@
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>Fase 5 — Streaming incremental completo (MLOps)</t>
+          <t>Fase 5 — Streaming incremental completo (rede e engajamento)</t>
         </is>
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>Scoring de persona online, Markov/IPED/Vamping incrementais — o sistema deixa de ser um relatório recalculado e passa a ser vivo.</t>
+          <t>Markov (persona e rede) e IPED/Vamping passam de agregação em lote para estado incremental por evento — persona não entra mais aqui, seu scoring incremental já roda desde a Fase 1. O sistema deixa de ser um relatório recalculado e passa a ser vivo.</t>
         </is>
       </c>
       <c r="D9" s="7" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E9" s="7" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="F9" s="8" t="inlineStr">
         <is>
           <t>Muito alto</t>
         </is>
       </c>
-      <c r="G9" s="11" t="inlineStr">
-        <is>
-          <t>Alto</t>
+      <c r="G9" s="9" t="inlineStr">
+        <is>
+          <t>Médio-Alto</t>
         </is>
       </c>
       <c r="H9" s="10">
-        <f>'Custo Detalhado'!G47</f>
+        <f>'Custo Detalhado'!G48</f>
         <v/>
       </c>
     </row>
@@ -883,75 +880,83 @@
         </is>
       </c>
       <c r="H10" s="10">
-        <f>'Custo Detalhado'!G56</f>
+        <f>'Custo Detalhado'!G57</f>
         <v/>
       </c>
     </row>
     <row r="11" ht="26" customHeight="1">
-      <c r="A11" s="12" t="inlineStr">
+      <c r="A11" s="11" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B11" s="12" t="n"/>
-      <c r="C11" s="12" t="n"/>
-      <c r="D11" s="12" t="n"/>
-      <c r="E11" s="12" t="n"/>
-      <c r="F11" s="12" t="n"/>
-      <c r="G11" s="12" t="n"/>
-      <c r="H11" s="13">
-        <f>'Custo Detalhado'!G58</f>
+      <c r="B11" s="11" t="n"/>
+      <c r="C11" s="11" t="n"/>
+      <c r="D11" s="11" t="n"/>
+      <c r="E11" s="11" t="n"/>
+      <c r="F11" s="11" t="n"/>
+      <c r="G11" s="11" t="n"/>
+      <c r="H11" s="12">
+        <f>'Custo Detalhado'!G59</f>
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="14" t="inlineStr">
+      <c r="A13" s="13" t="inlineStr">
         <is>
           <t>Notas de priorização</t>
         </is>
       </c>
     </row>
     <row r="14" ht="28" customHeight="1">
-      <c r="A14" s="15" t="inlineStr">
+      <c r="A14" s="14" t="inlineStr">
         <is>
           <t>• Fases 1 e 2 são as de melhor razão custo×benefício — nenhuma depende de integração nova de sistema, e reaproveitam a exportação de tensores e o motor de alarme que a CDRVIEW já tem em produção.</t>
         </is>
       </c>
     </row>
     <row r="15" ht="28" customHeight="1">
-      <c r="A15" s="15" t="inlineStr">
+      <c r="A15" s="14" t="inlineStr">
+        <is>
+          <t>• Persona (K-Means+XGBoost) entra na Fase 1 já no padrão real de produção da Claro — retreino trimestral batch + scoring semanal/incremental, dois jobs agendados sobre o tensor do CDRVIEW, sem esperar a infraestrutura de streaming da Fase 5.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="28" customHeight="1">
+      <c r="A16" s="14" t="inlineStr">
         <is>
           <t>• Fase 2 roda em paralelo à Fase 1 (equipes quase sem sobreposição) sem custo adicional de calendário.</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="28" customHeight="1">
-      <c r="A16" s="15" t="inlineStr">
+    <row r="17" ht="28" customHeight="1">
+      <c r="A17" s="14" t="inlineStr">
         <is>
           <t>• Fases 3 e 4 poderiam rodar em paralelo se um segundo Cientista de Dados Sênior for contratado (~R$28.000/mês adicional) — comprime o cronograma em ~4 sprints (8 semanas). Ver aba Cronograma.</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="28" customHeight="1">
-      <c r="A17" s="15" t="inlineStr">
-        <is>
-          <t>• Fase 5 (streaming/MLOps) é a mais cara e só compensa depois que as Fases 1, 3 e 4 já provaram valor em lote — evita re-trabalho de engenharia num modelo analítico ainda não validado pelo negócio.</t>
-        </is>
-      </c>
-    </row>
     <row r="18" ht="28" customHeight="1">
-      <c r="A18" s="15" t="inlineStr">
+      <c r="A18" s="14" t="inlineStr">
+        <is>
+          <t>• Fase 5 (streaming de rede/engajamento) é mais enxuta do que se persona estivesse incluída — só compensa depois que as Fases 2, 3 e 4 já provaram valor em lote, evitando re-trabalho de engenharia num modelo analítico ainda não validado pelo negócio.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="28" customHeight="1">
+      <c r="A19" s="14" t="inlineStr">
         <is>
           <t>• Custos de Rafael/Feijão/Andréia/CS são estimativas de alocação interna (custo de oportunidade), não gasto novo — mostrados para visibilidade total do custo do projeto, a validar com a Claro.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="8">
+  <mergeCells count="9">
     <mergeCell ref="A18:H18"/>
     <mergeCell ref="A15:H15"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A16:H16"/>
+    <mergeCell ref="A19:H19"/>
     <mergeCell ref="A14:H14"/>
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A11:G11"/>
@@ -1021,7 +1026,7 @@
           <t>PM / Coordenação geral</t>
         </is>
       </c>
-      <c r="B4" s="16" t="inlineStr">
+      <c r="B4" s="15" t="inlineStr">
         <is>
           <t>Vísent</t>
         </is>
@@ -1031,10 +1036,10 @@
           <t>Novo (contratado)</t>
         </is>
       </c>
-      <c r="D4" s="17" t="n">
+      <c r="D4" s="16" t="n">
         <v>30000</v>
       </c>
-      <c r="E4" s="18" t="inlineStr">
+      <c r="E4" s="17" t="inlineStr">
         <is>
           <t>Coordenação ponta a ponta entre Brintell, CDRVIEW e CS.</t>
         </is>
@@ -1046,7 +1051,7 @@
           <t>Arquiteto de Dados/Soluções Sênior</t>
         </is>
       </c>
-      <c r="B5" s="19" t="inlineStr">
+      <c r="B5" s="18" t="inlineStr">
         <is>
           <t>Brintell</t>
         </is>
@@ -1056,10 +1061,10 @@
           <t>Novo (contratado)</t>
         </is>
       </c>
-      <c r="D5" s="17" t="n">
+      <c r="D5" s="16" t="n">
         <v>33000</v>
       </c>
-      <c r="E5" s="18" t="inlineStr">
+      <c r="E5" s="17" t="inlineStr">
         <is>
           <t>Desenho de arquitetura, integração com os 4 tiers do CDRVIEW.</t>
         </is>
@@ -1071,7 +1076,7 @@
           <t>Engenheiro de Dados Sênior — Pipelines/Tensores</t>
         </is>
       </c>
-      <c r="B6" s="19" t="inlineStr">
+      <c r="B6" s="18" t="inlineStr">
         <is>
           <t>Brintell</t>
         </is>
@@ -1081,10 +1086,10 @@
           <t>Novo (contratado)</t>
         </is>
       </c>
-      <c r="D6" s="17" t="n">
+      <c r="D6" s="16" t="n">
         <v>27000</v>
       </c>
-      <c r="E6" s="18" t="inlineStr">
+      <c r="E6" s="17" t="inlineStr">
         <is>
           <t>Consome tensores 3D/4D já exportáveis pela GUI Análises do CDRVIEW.</t>
         </is>
@@ -1096,7 +1101,7 @@
           <t>Cientista de Dados Sênior — ML/Personas/Markov/Bayes</t>
         </is>
       </c>
-      <c r="B7" s="19" t="inlineStr">
+      <c r="B7" s="18" t="inlineStr">
         <is>
           <t>Brintell</t>
         </is>
@@ -1106,10 +1111,10 @@
           <t>Novo (contratado)</t>
         </is>
       </c>
-      <c r="D7" s="17" t="n">
+      <c r="D7" s="16" t="n">
         <v>28000</v>
       </c>
-      <c r="E7" s="18" t="inlineStr">
+      <c r="E7" s="17" t="inlineStr">
         <is>
           <t>K-Means/XGBoost, IPED, Vamping, Markov, Bayes ingênuo.</t>
         </is>
@@ -1121,7 +1126,7 @@
           <t>Engenheiro de Software Sênior — Dashboards/API</t>
         </is>
       </c>
-      <c r="B8" s="19" t="inlineStr">
+      <c r="B8" s="18" t="inlineStr">
         <is>
           <t>Brintell</t>
         </is>
@@ -1131,10 +1136,10 @@
           <t>Novo (contratado)</t>
         </is>
       </c>
-      <c r="D8" s="17" t="n">
+      <c r="D8" s="16" t="n">
         <v>25000</v>
       </c>
-      <c r="E8" s="18" t="inlineStr">
+      <c r="E8" s="17" t="inlineStr">
         <is>
           <t>Frontend consumidor de API (substitui o padrão de blob estático da PoC).</t>
         </is>
@@ -1146,7 +1151,7 @@
           <t>Engenheiro de Dados Sênior — MLOps/Streaming</t>
         </is>
       </c>
-      <c r="B9" s="19" t="inlineStr">
+      <c r="B9" s="18" t="inlineStr">
         <is>
           <t>Brintell</t>
         </is>
@@ -1156,10 +1161,10 @@
           <t>Novo (contratado)</t>
         </is>
       </c>
-      <c r="D9" s="17" t="n">
+      <c r="D9" s="16" t="n">
         <v>27000</v>
       </c>
-      <c r="E9" s="18" t="inlineStr">
+      <c r="E9" s="17" t="inlineStr">
         <is>
           <t>Incremental/online: scoring, Markov, IPED/Vamping incrementais (Fase 5).</t>
         </is>
@@ -1171,7 +1176,7 @@
           <t>Rafael — Eng. CDRVIEW Sênior (Parser/Ingestão/Redução/API)</t>
         </is>
       </c>
-      <c r="B10" s="16" t="inlineStr">
+      <c r="B10" s="15" t="inlineStr">
         <is>
           <t>Claro/CDRVIEW</t>
         </is>
@@ -1181,10 +1186,10 @@
           <t>Alocação interna (custo de oportunidade)</t>
         </is>
       </c>
-      <c r="D10" s="17" t="n">
+      <c r="D10" s="16" t="n">
         <v>28000</v>
       </c>
-      <c r="E10" s="18" t="inlineStr">
+      <c r="E10" s="17" t="inlineStr">
         <is>
           <t>Estimativa para dimensionar o projeto — não é gasto novo, é tempo já custeado pela Claro.</t>
         </is>
@@ -1196,7 +1201,7 @@
           <t>Feijão — Eng. CDRVIEW Sênior (Alarmística online/API)</t>
         </is>
       </c>
-      <c r="B11" s="16" t="inlineStr">
+      <c r="B11" s="15" t="inlineStr">
         <is>
           <t>Claro/CDRVIEW</t>
         </is>
@@ -1206,10 +1211,10 @@
           <t>Alocação interna (custo de oportunidade)</t>
         </is>
       </c>
-      <c r="D11" s="17" t="n">
+      <c r="D11" s="16" t="n">
         <v>28000</v>
       </c>
-      <c r="E11" s="18" t="inlineStr">
+      <c r="E11" s="17" t="inlineStr">
         <is>
           <t>Idem — estimativa de custo interno para visibilidade total do projeto.</t>
         </is>
@@ -1221,7 +1226,7 @@
           <t>Andréia — QA Sênior</t>
         </is>
       </c>
-      <c r="B12" s="16" t="inlineStr">
+      <c r="B12" s="15" t="inlineStr">
         <is>
           <t>Claro/CDRVIEW</t>
         </is>
@@ -1231,10 +1236,10 @@
           <t>Alocação interna (custo de oportunidade)</t>
         </is>
       </c>
-      <c r="D12" s="17" t="n">
+      <c r="D12" s="16" t="n">
         <v>18000</v>
       </c>
-      <c r="E12" s="18" t="inlineStr">
+      <c r="E12" s="17" t="inlineStr">
         <is>
           <t>Idem.</t>
         </is>
@@ -1246,7 +1251,7 @@
           <t>CS — Implantação/Rollout</t>
         </is>
       </c>
-      <c r="B13" s="16" t="inlineStr">
+      <c r="B13" s="15" t="inlineStr">
         <is>
           <t>Claro</t>
         </is>
@@ -1256,10 +1261,10 @@
           <t>Alocação interna (custo de oportunidade)</t>
         </is>
       </c>
-      <c r="D13" s="17" t="n">
+      <c r="D13" s="16" t="n">
         <v>20000</v>
       </c>
-      <c r="E13" s="18" t="inlineStr">
+      <c r="E13" s="17" t="inlineStr">
         <is>
           <t>Idem — líder de implantação, treinamento e go-live.</t>
         </is>
@@ -1279,7 +1284,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H58"/>
+  <dimension ref="A1:H59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -1360,16 +1365,16 @@
         </is>
       </c>
       <c r="C4" s="7" t="n">
-        <v>4</v>
-      </c>
-      <c r="D4" s="20">
+        <v>5</v>
+      </c>
+      <c r="D4" s="19">
         <f>C4*0.5</f>
         <v/>
       </c>
-      <c r="E4" s="21" t="n">
+      <c r="E4" s="20" t="n">
         <v>0.5</v>
       </c>
-      <c r="F4" s="17">
+      <c r="F4" s="16">
         <f>Papéis!D4</f>
         <v/>
       </c>
@@ -1377,7 +1382,7 @@
         <f>D4*E4*F4</f>
         <v/>
       </c>
-      <c r="H4" s="16">
+      <c r="H4" s="15">
         <f>Papéis!B4</f>
         <v/>
       </c>
@@ -1394,16 +1399,16 @@
         </is>
       </c>
       <c r="C5" s="7" t="n">
-        <v>4</v>
-      </c>
-      <c r="D5" s="20">
+        <v>5</v>
+      </c>
+      <c r="D5" s="19">
         <f>C5*0.5</f>
         <v/>
       </c>
-      <c r="E5" s="21" t="n">
+      <c r="E5" s="20" t="n">
         <v>0.5</v>
       </c>
-      <c r="F5" s="17">
+      <c r="F5" s="16">
         <f>Papéis!D5</f>
         <v/>
       </c>
@@ -1411,7 +1416,7 @@
         <f>D5*E5*F5</f>
         <v/>
       </c>
-      <c r="H5" s="19">
+      <c r="H5" s="18">
         <f>Papéis!B5</f>
         <v/>
       </c>
@@ -1428,16 +1433,16 @@
         </is>
       </c>
       <c r="C6" s="7" t="n">
-        <v>4</v>
-      </c>
-      <c r="D6" s="20">
+        <v>5</v>
+      </c>
+      <c r="D6" s="19">
         <f>C6*0.5</f>
         <v/>
       </c>
-      <c r="E6" s="21" t="n">
+      <c r="E6" s="20" t="n">
         <v>1</v>
       </c>
-      <c r="F6" s="17">
+      <c r="F6" s="16">
         <f>Papéis!D6</f>
         <v/>
       </c>
@@ -1445,7 +1450,7 @@
         <f>D6*E6*F6</f>
         <v/>
       </c>
-      <c r="H6" s="19">
+      <c r="H6" s="18">
         <f>Papéis!B6</f>
         <v/>
       </c>
@@ -1462,16 +1467,16 @@
         </is>
       </c>
       <c r="C7" s="7" t="n">
-        <v>4</v>
-      </c>
-      <c r="D7" s="20">
+        <v>5</v>
+      </c>
+      <c r="D7" s="19">
         <f>C7*0.5</f>
         <v/>
       </c>
-      <c r="E7" s="21" t="n">
+      <c r="E7" s="20" t="n">
         <v>1</v>
       </c>
-      <c r="F7" s="17">
+      <c r="F7" s="16">
         <f>Papéis!D7</f>
         <v/>
       </c>
@@ -1479,7 +1484,7 @@
         <f>D7*E7*F7</f>
         <v/>
       </c>
-      <c r="H7" s="19">
+      <c r="H7" s="18">
         <f>Papéis!B7</f>
         <v/>
       </c>
@@ -1496,16 +1501,16 @@
         </is>
       </c>
       <c r="C8" s="7" t="n">
-        <v>4</v>
-      </c>
-      <c r="D8" s="20">
+        <v>5</v>
+      </c>
+      <c r="D8" s="19">
         <f>C8*0.5</f>
         <v/>
       </c>
-      <c r="E8" s="21" t="n">
+      <c r="E8" s="20" t="n">
         <v>0.5</v>
       </c>
-      <c r="F8" s="17">
+      <c r="F8" s="16">
         <f>Papéis!D8</f>
         <v/>
       </c>
@@ -1513,7 +1518,7 @@
         <f>D8*E8*F8</f>
         <v/>
       </c>
-      <c r="H8" s="19">
+      <c r="H8" s="18">
         <f>Papéis!B8</f>
         <v/>
       </c>
@@ -1526,29 +1531,29 @@
       </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>Rafael — Eng. CDRVIEW Sênior (Parser/Ingestão/Redução/API)</t>
+          <t>Engenheiro de Dados Sênior — MLOps/Streaming</t>
         </is>
       </c>
       <c r="C9" s="7" t="n">
-        <v>4</v>
-      </c>
-      <c r="D9" s="20">
+        <v>5</v>
+      </c>
+      <c r="D9" s="19">
         <f>C9*0.5</f>
         <v/>
       </c>
-      <c r="E9" s="21" t="n">
+      <c r="E9" s="20" t="n">
         <v>0.2</v>
       </c>
-      <c r="F9" s="17">
-        <f>Papéis!D10</f>
+      <c r="F9" s="16">
+        <f>Papéis!D9</f>
         <v/>
       </c>
       <c r="G9" s="10">
         <f>D9*E9*F9</f>
         <v/>
       </c>
-      <c r="H9" s="16">
-        <f>Papéis!B10</f>
+      <c r="H9" s="18">
+        <f>Papéis!B9</f>
         <v/>
       </c>
     </row>
@@ -1560,29 +1565,29 @@
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>Andréia — QA Sênior</t>
+          <t>Rafael — Eng. CDRVIEW Sênior (Parser/Ingestão/Redução/API)</t>
         </is>
       </c>
       <c r="C10" s="7" t="n">
-        <v>4</v>
-      </c>
-      <c r="D10" s="20">
+        <v>5</v>
+      </c>
+      <c r="D10" s="19">
         <f>C10*0.5</f>
         <v/>
       </c>
-      <c r="E10" s="21" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="F10" s="17">
-        <f>Papéis!D12</f>
+      <c r="E10" s="20" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F10" s="16">
+        <f>Papéis!D10</f>
         <v/>
       </c>
       <c r="G10" s="10">
         <f>D10*E10*F10</f>
         <v/>
       </c>
-      <c r="H10" s="16">
-        <f>Papéis!B12</f>
+      <c r="H10" s="15">
+        <f>Papéis!B10</f>
         <v/>
       </c>
     </row>
@@ -1594,82 +1599,82 @@
       </c>
       <c r="B11" s="7" t="inlineStr">
         <is>
-          <t>CS — Implantação/Rollout</t>
+          <t>Andréia — QA Sênior</t>
         </is>
       </c>
       <c r="C11" s="7" t="n">
-        <v>4</v>
-      </c>
-      <c r="D11" s="20">
+        <v>5</v>
+      </c>
+      <c r="D11" s="19">
         <f>C11*0.5</f>
         <v/>
       </c>
-      <c r="E11" s="21" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="F11" s="17">
-        <f>Papéis!D13</f>
+      <c r="E11" s="20" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F11" s="16">
+        <f>Papéis!D12</f>
         <v/>
       </c>
       <c r="G11" s="10">
         <f>D11*E11*F11</f>
         <v/>
       </c>
-      <c r="H11" s="16">
+      <c r="H11" s="15">
+        <f>Papéis!B12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>Fase 1 — Personas &amp; Qualidade de Deslocamento</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>CS — Implantação/Rollout</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="D12" s="19">
+        <f>C12*0.5</f>
+        <v/>
+      </c>
+      <c r="E12" s="20" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F12" s="16">
+        <f>Papéis!D13</f>
+        <v/>
+      </c>
+      <c r="G12" s="10">
+        <f>D12*E12*F12</f>
+        <v/>
+      </c>
+      <c r="H12" s="15">
         <f>Papéis!B13</f>
         <v/>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="22" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="21" t="inlineStr">
         <is>
           <t>Subtotal — Fase 1 — Personas &amp; Qualidade de Deslocamento</t>
         </is>
       </c>
-      <c r="B12" s="23" t="n"/>
-      <c r="C12" s="23" t="n"/>
-      <c r="D12" s="23" t="n"/>
-      <c r="E12" s="23" t="n"/>
-      <c r="F12" s="23" t="n"/>
-      <c r="G12" s="24">
-        <f>SUM(G4:G11)</f>
-        <v/>
-      </c>
-      <c r="H12" s="23" t="n"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="7" t="inlineStr">
-        <is>
-          <t>Fase 2 — Dashboard da Alarmística existente</t>
-        </is>
-      </c>
-      <c r="B14" s="7" t="inlineStr">
-        <is>
-          <t>PM / Coordenação geral</t>
-        </is>
-      </c>
-      <c r="C14" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="D14" s="20">
-        <f>C14*0.5</f>
-        <v/>
-      </c>
-      <c r="E14" s="21" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="F14" s="17">
-        <f>Papéis!D4</f>
-        <v/>
-      </c>
-      <c r="G14" s="10">
-        <f>D14*E14*F14</f>
-        <v/>
-      </c>
-      <c r="H14" s="16">
-        <f>Papéis!B4</f>
-        <v/>
-      </c>
+      <c r="B13" s="22" t="n"/>
+      <c r="C13" s="22" t="n"/>
+      <c r="D13" s="22" t="n"/>
+      <c r="E13" s="22" t="n"/>
+      <c r="F13" s="22" t="n"/>
+      <c r="G13" s="23">
+        <f>SUM(G4:G12)</f>
+        <v/>
+      </c>
+      <c r="H13" s="22" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
@@ -1679,29 +1684,29 @@
       </c>
       <c r="B15" s="7" t="inlineStr">
         <is>
-          <t>Engenheiro de Software Sênior — Dashboards/API</t>
+          <t>PM / Coordenação geral</t>
         </is>
       </c>
       <c r="C15" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="D15" s="20">
+      <c r="D15" s="19">
         <f>C15*0.5</f>
         <v/>
       </c>
-      <c r="E15" s="21" t="n">
-        <v>1</v>
-      </c>
-      <c r="F15" s="17">
-        <f>Papéis!D8</f>
+      <c r="E15" s="20" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F15" s="16">
+        <f>Papéis!D4</f>
         <v/>
       </c>
       <c r="G15" s="10">
         <f>D15*E15*F15</f>
         <v/>
       </c>
-      <c r="H15" s="19">
-        <f>Papéis!B8</f>
+      <c r="H15" s="15">
+        <f>Papéis!B4</f>
         <v/>
       </c>
     </row>
@@ -1713,29 +1718,29 @@
       </c>
       <c r="B16" s="7" t="inlineStr">
         <is>
-          <t>Feijão — Eng. CDRVIEW Sênior (Alarmística online/API)</t>
+          <t>Engenheiro de Software Sênior — Dashboards/API</t>
         </is>
       </c>
       <c r="C16" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="D16" s="20">
+      <c r="D16" s="19">
         <f>C16*0.5</f>
         <v/>
       </c>
-      <c r="E16" s="21" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="F16" s="17">
-        <f>Papéis!D11</f>
+      <c r="E16" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="F16" s="16">
+        <f>Papéis!D8</f>
         <v/>
       </c>
       <c r="G16" s="10">
         <f>D16*E16*F16</f>
         <v/>
       </c>
-      <c r="H16" s="16">
-        <f>Papéis!B11</f>
+      <c r="H16" s="18">
+        <f>Papéis!B8</f>
         <v/>
       </c>
     </row>
@@ -1747,82 +1752,82 @@
       </c>
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>Andréia — QA Sênior</t>
+          <t>Feijão — Eng. CDRVIEW Sênior (Alarmística online/API)</t>
         </is>
       </c>
       <c r="C17" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="D17" s="20">
+      <c r="D17" s="19">
         <f>C17*0.5</f>
         <v/>
       </c>
-      <c r="E17" s="21" t="n">
+      <c r="E17" s="20" t="n">
         <v>0.3</v>
       </c>
-      <c r="F17" s="17">
-        <f>Papéis!D12</f>
+      <c r="F17" s="16">
+        <f>Papéis!D11</f>
         <v/>
       </c>
       <c r="G17" s="10">
         <f>D17*E17*F17</f>
         <v/>
       </c>
-      <c r="H17" s="16">
+      <c r="H17" s="15">
+        <f>Papéis!B11</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="7" t="inlineStr">
+        <is>
+          <t>Fase 2 — Dashboard da Alarmística existente</t>
+        </is>
+      </c>
+      <c r="B18" s="7" t="inlineStr">
+        <is>
+          <t>Andréia — QA Sênior</t>
+        </is>
+      </c>
+      <c r="C18" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D18" s="19">
+        <f>C18*0.5</f>
+        <v/>
+      </c>
+      <c r="E18" s="20" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F18" s="16">
+        <f>Papéis!D12</f>
+        <v/>
+      </c>
+      <c r="G18" s="10">
+        <f>D18*E18*F18</f>
+        <v/>
+      </c>
+      <c r="H18" s="15">
         <f>Papéis!B12</f>
         <v/>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="22" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="21" t="inlineStr">
         <is>
           <t>Subtotal — Fase 2 — Dashboard da Alarmística existente</t>
         </is>
       </c>
-      <c r="B18" s="23" t="n"/>
-      <c r="C18" s="23" t="n"/>
-      <c r="D18" s="23" t="n"/>
-      <c r="E18" s="23" t="n"/>
-      <c r="F18" s="23" t="n"/>
-      <c r="G18" s="24">
-        <f>SUM(G14:G17)</f>
-        <v/>
-      </c>
-      <c r="H18" s="23" t="n"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="7" t="inlineStr">
-        <is>
-          <t>Fase 3 — Analytics novo sobre a Alarmística</t>
-        </is>
-      </c>
-      <c r="B20" s="7" t="inlineStr">
-        <is>
-          <t>PM / Coordenação geral</t>
-        </is>
-      </c>
-      <c r="C20" s="7" t="n">
-        <v>3</v>
-      </c>
-      <c r="D20" s="20">
-        <f>C20*0.5</f>
-        <v/>
-      </c>
-      <c r="E20" s="21" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="F20" s="17">
-        <f>Papéis!D4</f>
-        <v/>
-      </c>
-      <c r="G20" s="10">
-        <f>D20*E20*F20</f>
-        <v/>
-      </c>
-      <c r="H20" s="16">
-        <f>Papéis!B4</f>
-        <v/>
-      </c>
+      <c r="B19" s="22" t="n"/>
+      <c r="C19" s="22" t="n"/>
+      <c r="D19" s="22" t="n"/>
+      <c r="E19" s="22" t="n"/>
+      <c r="F19" s="22" t="n"/>
+      <c r="G19" s="23">
+        <f>SUM(G15:G18)</f>
+        <v/>
+      </c>
+      <c r="H19" s="22" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="7" t="inlineStr">
@@ -1832,29 +1837,29 @@
       </c>
       <c r="B21" s="7" t="inlineStr">
         <is>
-          <t>Arquiteto de Dados/Soluções Sênior</t>
+          <t>PM / Coordenação geral</t>
         </is>
       </c>
       <c r="C21" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="D21" s="20">
+      <c r="D21" s="19">
         <f>C21*0.5</f>
         <v/>
       </c>
-      <c r="E21" s="21" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="F21" s="17">
-        <f>Papéis!D5</f>
+      <c r="E21" s="20" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F21" s="16">
+        <f>Papéis!D4</f>
         <v/>
       </c>
       <c r="G21" s="10">
         <f>D21*E21*F21</f>
         <v/>
       </c>
-      <c r="H21" s="19">
-        <f>Papéis!B5</f>
+      <c r="H21" s="15">
+        <f>Papéis!B4</f>
         <v/>
       </c>
     </row>
@@ -1866,29 +1871,29 @@
       </c>
       <c r="B22" s="7" t="inlineStr">
         <is>
-          <t>Cientista de Dados Sênior — ML/Personas/Markov/Bayes</t>
+          <t>Arquiteto de Dados/Soluções Sênior</t>
         </is>
       </c>
       <c r="C22" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="D22" s="20">
+      <c r="D22" s="19">
         <f>C22*0.5</f>
         <v/>
       </c>
-      <c r="E22" s="21" t="n">
-        <v>1</v>
-      </c>
-      <c r="F22" s="17">
-        <f>Papéis!D7</f>
+      <c r="E22" s="20" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F22" s="16">
+        <f>Papéis!D5</f>
         <v/>
       </c>
       <c r="G22" s="10">
         <f>D22*E22*F22</f>
         <v/>
       </c>
-      <c r="H22" s="19">
-        <f>Papéis!B7</f>
+      <c r="H22" s="18">
+        <f>Papéis!B5</f>
         <v/>
       </c>
     </row>
@@ -1900,29 +1905,29 @@
       </c>
       <c r="B23" s="7" t="inlineStr">
         <is>
-          <t>Engenheiro de Software Sênior — Dashboards/API</t>
+          <t>Cientista de Dados Sênior — ML/Personas/Markov/Bayes</t>
         </is>
       </c>
       <c r="C23" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="D23" s="20">
+      <c r="D23" s="19">
         <f>C23*0.5</f>
         <v/>
       </c>
-      <c r="E23" s="21" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="F23" s="17">
-        <f>Papéis!D8</f>
+      <c r="E23" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="F23" s="16">
+        <f>Papéis!D7</f>
         <v/>
       </c>
       <c r="G23" s="10">
         <f>D23*E23*F23</f>
         <v/>
       </c>
-      <c r="H23" s="19">
-        <f>Papéis!B8</f>
+      <c r="H23" s="18">
+        <f>Papéis!B7</f>
         <v/>
       </c>
     </row>
@@ -1934,29 +1939,29 @@
       </c>
       <c r="B24" s="7" t="inlineStr">
         <is>
-          <t>Feijão — Eng. CDRVIEW Sênior (Alarmística online/API)</t>
+          <t>Engenheiro de Software Sênior — Dashboards/API</t>
         </is>
       </c>
       <c r="C24" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="D24" s="20">
+      <c r="D24" s="19">
         <f>C24*0.5</f>
         <v/>
       </c>
-      <c r="E24" s="21" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="F24" s="17">
-        <f>Papéis!D11</f>
+      <c r="E24" s="20" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F24" s="16">
+        <f>Papéis!D8</f>
         <v/>
       </c>
       <c r="G24" s="10">
         <f>D24*E24*F24</f>
         <v/>
       </c>
-      <c r="H24" s="16">
-        <f>Papéis!B11</f>
+      <c r="H24" s="18">
+        <f>Papéis!B8</f>
         <v/>
       </c>
     </row>
@@ -1968,82 +1973,82 @@
       </c>
       <c r="B25" s="7" t="inlineStr">
         <is>
-          <t>Andréia — QA Sênior</t>
+          <t>Feijão — Eng. CDRVIEW Sênior (Alarmística online/API)</t>
         </is>
       </c>
       <c r="C25" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="D25" s="20">
+      <c r="D25" s="19">
         <f>C25*0.5</f>
         <v/>
       </c>
-      <c r="E25" s="21" t="n">
+      <c r="E25" s="20" t="n">
         <v>0.3</v>
       </c>
-      <c r="F25" s="17">
-        <f>Papéis!D12</f>
+      <c r="F25" s="16">
+        <f>Papéis!D11</f>
         <v/>
       </c>
       <c r="G25" s="10">
         <f>D25*E25*F25</f>
         <v/>
       </c>
-      <c r="H25" s="16">
+      <c r="H25" s="15">
+        <f>Papéis!B11</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="7" t="inlineStr">
+        <is>
+          <t>Fase 3 — Analytics novo sobre a Alarmística</t>
+        </is>
+      </c>
+      <c r="B26" s="7" t="inlineStr">
+        <is>
+          <t>Andréia — QA Sênior</t>
+        </is>
+      </c>
+      <c r="C26" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="D26" s="19">
+        <f>C26*0.5</f>
+        <v/>
+      </c>
+      <c r="E26" s="20" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F26" s="16">
+        <f>Papéis!D12</f>
+        <v/>
+      </c>
+      <c r="G26" s="10">
+        <f>D26*E26*F26</f>
+        <v/>
+      </c>
+      <c r="H26" s="15">
         <f>Papéis!B12</f>
         <v/>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="22" t="inlineStr">
+    <row r="27">
+      <c r="A27" s="21" t="inlineStr">
         <is>
           <t>Subtotal — Fase 3 — Analytics novo sobre a Alarmística</t>
         </is>
       </c>
-      <c r="B26" s="23" t="n"/>
-      <c r="C26" s="23" t="n"/>
-      <c r="D26" s="23" t="n"/>
-      <c r="E26" s="23" t="n"/>
-      <c r="F26" s="23" t="n"/>
-      <c r="G26" s="24">
-        <f>SUM(G20:G25)</f>
-        <v/>
-      </c>
-      <c r="H26" s="23" t="n"/>
-    </row>
-    <row r="28">
-      <c r="A28" s="7" t="inlineStr">
-        <is>
-          <t>Fase 4 — Topologia de rede + Priorização de alertas</t>
-        </is>
-      </c>
-      <c r="B28" s="7" t="inlineStr">
-        <is>
-          <t>PM / Coordenação geral</t>
-        </is>
-      </c>
-      <c r="C28" s="7" t="n">
-        <v>4</v>
-      </c>
-      <c r="D28" s="20">
-        <f>C28*0.5</f>
-        <v/>
-      </c>
-      <c r="E28" s="21" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="F28" s="17">
-        <f>Papéis!D4</f>
-        <v/>
-      </c>
-      <c r="G28" s="10">
-        <f>D28*E28*F28</f>
-        <v/>
-      </c>
-      <c r="H28" s="16">
-        <f>Papéis!B4</f>
-        <v/>
-      </c>
+      <c r="B27" s="22" t="n"/>
+      <c r="C27" s="22" t="n"/>
+      <c r="D27" s="22" t="n"/>
+      <c r="E27" s="22" t="n"/>
+      <c r="F27" s="22" t="n"/>
+      <c r="G27" s="23">
+        <f>SUM(G21:G26)</f>
+        <v/>
+      </c>
+      <c r="H27" s="22" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="7" t="inlineStr">
@@ -2053,29 +2058,29 @@
       </c>
       <c r="B29" s="7" t="inlineStr">
         <is>
-          <t>Arquiteto de Dados/Soluções Sênior</t>
+          <t>PM / Coordenação geral</t>
         </is>
       </c>
       <c r="C29" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="D29" s="20">
+      <c r="D29" s="19">
         <f>C29*0.5</f>
         <v/>
       </c>
-      <c r="E29" s="21" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="F29" s="17">
-        <f>Papéis!D5</f>
+      <c r="E29" s="20" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="F29" s="16">
+        <f>Papéis!D4</f>
         <v/>
       </c>
       <c r="G29" s="10">
         <f>D29*E29*F29</f>
         <v/>
       </c>
-      <c r="H29" s="19">
-        <f>Papéis!B5</f>
+      <c r="H29" s="15">
+        <f>Papéis!B4</f>
         <v/>
       </c>
     </row>
@@ -2087,29 +2092,29 @@
       </c>
       <c r="B30" s="7" t="inlineStr">
         <is>
-          <t>Engenheiro de Dados Sênior — Pipelines/Tensores</t>
+          <t>Arquiteto de Dados/Soluções Sênior</t>
         </is>
       </c>
       <c r="C30" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="D30" s="20">
+      <c r="D30" s="19">
         <f>C30*0.5</f>
         <v/>
       </c>
-      <c r="E30" s="21" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="F30" s="17">
-        <f>Papéis!D6</f>
+      <c r="E30" s="20" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F30" s="16">
+        <f>Papéis!D5</f>
         <v/>
       </c>
       <c r="G30" s="10">
         <f>D30*E30*F30</f>
         <v/>
       </c>
-      <c r="H30" s="19">
-        <f>Papéis!B6</f>
+      <c r="H30" s="18">
+        <f>Papéis!B5</f>
         <v/>
       </c>
     </row>
@@ -2121,29 +2126,29 @@
       </c>
       <c r="B31" s="7" t="inlineStr">
         <is>
-          <t>Cientista de Dados Sênior — ML/Personas/Markov/Bayes</t>
+          <t>Engenheiro de Dados Sênior — Pipelines/Tensores</t>
         </is>
       </c>
       <c r="C31" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="D31" s="20">
+      <c r="D31" s="19">
         <f>C31*0.5</f>
         <v/>
       </c>
-      <c r="E31" s="21" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="F31" s="17">
-        <f>Papéis!D7</f>
+      <c r="E31" s="20" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="F31" s="16">
+        <f>Papéis!D6</f>
         <v/>
       </c>
       <c r="G31" s="10">
         <f>D31*E31*F31</f>
         <v/>
       </c>
-      <c r="H31" s="19">
-        <f>Papéis!B7</f>
+      <c r="H31" s="18">
+        <f>Papéis!B6</f>
         <v/>
       </c>
     </row>
@@ -2155,29 +2160,29 @@
       </c>
       <c r="B32" s="7" t="inlineStr">
         <is>
-          <t>Engenheiro de Software Sênior — Dashboards/API</t>
+          <t>Cientista de Dados Sênior — ML/Personas/Markov/Bayes</t>
         </is>
       </c>
       <c r="C32" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="D32" s="20">
+      <c r="D32" s="19">
         <f>C32*0.5</f>
         <v/>
       </c>
-      <c r="E32" s="21" t="n">
+      <c r="E32" s="20" t="n">
         <v>0.6</v>
       </c>
-      <c r="F32" s="17">
-        <f>Papéis!D8</f>
+      <c r="F32" s="16">
+        <f>Papéis!D7</f>
         <v/>
       </c>
       <c r="G32" s="10">
         <f>D32*E32*F32</f>
         <v/>
       </c>
-      <c r="H32" s="19">
-        <f>Papéis!B8</f>
+      <c r="H32" s="18">
+        <f>Papéis!B7</f>
         <v/>
       </c>
     </row>
@@ -2189,29 +2194,29 @@
       </c>
       <c r="B33" s="7" t="inlineStr">
         <is>
-          <t>Rafael — Eng. CDRVIEW Sênior (Parser/Ingestão/Redução/API)</t>
+          <t>Engenheiro de Software Sênior — Dashboards/API</t>
         </is>
       </c>
       <c r="C33" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="D33" s="20">
+      <c r="D33" s="19">
         <f>C33*0.5</f>
         <v/>
       </c>
-      <c r="E33" s="21" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="F33" s="17">
-        <f>Papéis!D10</f>
+      <c r="E33" s="20" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="F33" s="16">
+        <f>Papéis!D8</f>
         <v/>
       </c>
       <c r="G33" s="10">
         <f>D33*E33*F33</f>
         <v/>
       </c>
-      <c r="H33" s="16">
-        <f>Papéis!B10</f>
+      <c r="H33" s="18">
+        <f>Papéis!B8</f>
         <v/>
       </c>
     </row>
@@ -2223,29 +2228,29 @@
       </c>
       <c r="B34" s="7" t="inlineStr">
         <is>
-          <t>Andréia — QA Sênior</t>
+          <t>Rafael — Eng. CDRVIEW Sênior (Parser/Ingestão/Redução/API)</t>
         </is>
       </c>
       <c r="C34" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="D34" s="20">
+      <c r="D34" s="19">
         <f>C34*0.5</f>
         <v/>
       </c>
-      <c r="E34" s="21" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="F34" s="17">
-        <f>Papéis!D12</f>
+      <c r="E34" s="20" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F34" s="16">
+        <f>Papéis!D10</f>
         <v/>
       </c>
       <c r="G34" s="10">
         <f>D34*E34*F34</f>
         <v/>
       </c>
-      <c r="H34" s="16">
-        <f>Papéis!B12</f>
+      <c r="H34" s="15">
+        <f>Papéis!B10</f>
         <v/>
       </c>
     </row>
@@ -2257,405 +2262,405 @@
       </c>
       <c r="B35" s="7" t="inlineStr">
         <is>
-          <t>CS — Implantação/Rollout</t>
+          <t>Andréia — QA Sênior</t>
         </is>
       </c>
       <c r="C35" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="D35" s="20">
+      <c r="D35" s="19">
         <f>C35*0.5</f>
         <v/>
       </c>
-      <c r="E35" s="21" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="F35" s="17">
-        <f>Papéis!D13</f>
+      <c r="E35" s="20" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="F35" s="16">
+        <f>Papéis!D12</f>
         <v/>
       </c>
       <c r="G35" s="10">
         <f>D35*E35*F35</f>
         <v/>
       </c>
-      <c r="H35" s="16">
+      <c r="H35" s="15">
+        <f>Papéis!B12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="7" t="inlineStr">
+        <is>
+          <t>Fase 4 — Topologia de rede + Priorização de alertas</t>
+        </is>
+      </c>
+      <c r="B36" s="7" t="inlineStr">
+        <is>
+          <t>CS — Implantação/Rollout</t>
+        </is>
+      </c>
+      <c r="C36" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="D36" s="19">
+        <f>C36*0.5</f>
+        <v/>
+      </c>
+      <c r="E36" s="20" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F36" s="16">
+        <f>Papéis!D13</f>
+        <v/>
+      </c>
+      <c r="G36" s="10">
+        <f>D36*E36*F36</f>
+        <v/>
+      </c>
+      <c r="H36" s="15">
         <f>Papéis!B13</f>
         <v/>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="22" t="inlineStr">
+    <row r="37">
+      <c r="A37" s="21" t="inlineStr">
         <is>
           <t>Subtotal — Fase 4 — Topologia de rede + Priorização de alertas</t>
         </is>
       </c>
-      <c r="B36" s="23" t="n"/>
-      <c r="C36" s="23" t="n"/>
-      <c r="D36" s="23" t="n"/>
-      <c r="E36" s="23" t="n"/>
-      <c r="F36" s="23" t="n"/>
-      <c r="G36" s="24">
-        <f>SUM(G28:G35)</f>
-        <v/>
-      </c>
-      <c r="H36" s="23" t="n"/>
-    </row>
-    <row r="38">
-      <c r="A38" s="7" t="inlineStr">
-        <is>
-          <t>Fase 5 — Streaming incremental completo (MLOps)</t>
-        </is>
-      </c>
-      <c r="B38" s="7" t="inlineStr">
-        <is>
-          <t>PM / Coordenação geral</t>
-        </is>
-      </c>
-      <c r="C38" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="D38" s="20">
-        <f>C38*0.5</f>
-        <v/>
-      </c>
-      <c r="E38" s="21" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="F38" s="17">
-        <f>Papéis!D4</f>
-        <v/>
-      </c>
-      <c r="G38" s="10">
-        <f>D38*E38*F38</f>
-        <v/>
-      </c>
-      <c r="H38" s="16">
-        <f>Papéis!B4</f>
-        <v/>
-      </c>
+      <c r="B37" s="22" t="n"/>
+      <c r="C37" s="22" t="n"/>
+      <c r="D37" s="22" t="n"/>
+      <c r="E37" s="22" t="n"/>
+      <c r="F37" s="22" t="n"/>
+      <c r="G37" s="23">
+        <f>SUM(G29:G36)</f>
+        <v/>
+      </c>
+      <c r="H37" s="22" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="7" t="inlineStr">
         <is>
-          <t>Fase 5 — Streaming incremental completo (MLOps)</t>
+          <t>Fase 5 — Streaming incremental completo (rede e engajamento)</t>
         </is>
       </c>
       <c r="B39" s="7" t="inlineStr">
         <is>
-          <t>Arquiteto de Dados/Soluções Sênior</t>
+          <t>PM / Coordenação geral</t>
         </is>
       </c>
       <c r="C39" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="D39" s="20">
+        <v>5</v>
+      </c>
+      <c r="D39" s="19">
         <f>C39*0.5</f>
         <v/>
       </c>
-      <c r="E39" s="21" t="n">
+      <c r="E39" s="20" t="n">
         <v>0.5</v>
       </c>
-      <c r="F39" s="17">
-        <f>Papéis!D5</f>
+      <c r="F39" s="16">
+        <f>Papéis!D4</f>
         <v/>
       </c>
       <c r="G39" s="10">
         <f>D39*E39*F39</f>
         <v/>
       </c>
-      <c r="H39" s="19">
-        <f>Papéis!B5</f>
+      <c r="H39" s="15">
+        <f>Papéis!B4</f>
         <v/>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="7" t="inlineStr">
         <is>
-          <t>Fase 5 — Streaming incremental completo (MLOps)</t>
+          <t>Fase 5 — Streaming incremental completo (rede e engajamento)</t>
         </is>
       </c>
       <c r="B40" s="7" t="inlineStr">
         <is>
-          <t>Cientista de Dados Sênior — ML/Personas/Markov/Bayes</t>
+          <t>Arquiteto de Dados/Soluções Sênior</t>
         </is>
       </c>
       <c r="C40" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="D40" s="20">
+        <v>5</v>
+      </c>
+      <c r="D40" s="19">
         <f>C40*0.5</f>
         <v/>
       </c>
-      <c r="E40" s="21" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="F40" s="17">
-        <f>Papéis!D7</f>
+      <c r="E40" s="20" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F40" s="16">
+        <f>Papéis!D5</f>
         <v/>
       </c>
       <c r="G40" s="10">
         <f>D40*E40*F40</f>
         <v/>
       </c>
-      <c r="H40" s="19">
-        <f>Papéis!B7</f>
+      <c r="H40" s="18">
+        <f>Papéis!B5</f>
         <v/>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="7" t="inlineStr">
         <is>
-          <t>Fase 5 — Streaming incremental completo (MLOps)</t>
+          <t>Fase 5 — Streaming incremental completo (rede e engajamento)</t>
         </is>
       </c>
       <c r="B41" s="7" t="inlineStr">
         <is>
-          <t>Engenheiro de Software Sênior — Dashboards/API</t>
+          <t>Cientista de Dados Sênior — ML/Personas/Markov/Bayes</t>
         </is>
       </c>
       <c r="C41" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="D41" s="20">
+        <v>5</v>
+      </c>
+      <c r="D41" s="19">
         <f>C41*0.5</f>
         <v/>
       </c>
-      <c r="E41" s="21" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="F41" s="17">
-        <f>Papéis!D8</f>
+      <c r="E41" s="20" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="F41" s="16">
+        <f>Papéis!D7</f>
         <v/>
       </c>
       <c r="G41" s="10">
         <f>D41*E41*F41</f>
         <v/>
       </c>
-      <c r="H41" s="19">
-        <f>Papéis!B8</f>
+      <c r="H41" s="18">
+        <f>Papéis!B7</f>
         <v/>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="7" t="inlineStr">
         <is>
-          <t>Fase 5 — Streaming incremental completo (MLOps)</t>
+          <t>Fase 5 — Streaming incremental completo (rede e engajamento)</t>
         </is>
       </c>
       <c r="B42" s="7" t="inlineStr">
         <is>
-          <t>Engenheiro de Dados Sênior — MLOps/Streaming</t>
+          <t>Engenheiro de Software Sênior — Dashboards/API</t>
         </is>
       </c>
       <c r="C42" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="D42" s="20">
+        <v>5</v>
+      </c>
+      <c r="D42" s="19">
         <f>C42*0.5</f>
         <v/>
       </c>
-      <c r="E42" s="21" t="n">
-        <v>1</v>
-      </c>
-      <c r="F42" s="17">
-        <f>Papéis!D9</f>
+      <c r="E42" s="20" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F42" s="16">
+        <f>Papéis!D8</f>
         <v/>
       </c>
       <c r="G42" s="10">
         <f>D42*E42*F42</f>
         <v/>
       </c>
-      <c r="H42" s="19">
-        <f>Papéis!B9</f>
+      <c r="H42" s="18">
+        <f>Papéis!B8</f>
         <v/>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="7" t="inlineStr">
         <is>
-          <t>Fase 5 — Streaming incremental completo (MLOps)</t>
+          <t>Fase 5 — Streaming incremental completo (rede e engajamento)</t>
         </is>
       </c>
       <c r="B43" s="7" t="inlineStr">
         <is>
-          <t>Rafael — Eng. CDRVIEW Sênior (Parser/Ingestão/Redução/API)</t>
+          <t>Engenheiro de Dados Sênior — MLOps/Streaming</t>
         </is>
       </c>
       <c r="C43" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="D43" s="20">
+        <v>5</v>
+      </c>
+      <c r="D43" s="19">
         <f>C43*0.5</f>
         <v/>
       </c>
-      <c r="E43" s="21" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="F43" s="17">
-        <f>Papéis!D10</f>
+      <c r="E43" s="20" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="F43" s="16">
+        <f>Papéis!D9</f>
         <v/>
       </c>
       <c r="G43" s="10">
         <f>D43*E43*F43</f>
         <v/>
       </c>
-      <c r="H43" s="16">
-        <f>Papéis!B10</f>
+      <c r="H43" s="18">
+        <f>Papéis!B9</f>
         <v/>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="7" t="inlineStr">
         <is>
-          <t>Fase 5 — Streaming incremental completo (MLOps)</t>
+          <t>Fase 5 — Streaming incremental completo (rede e engajamento)</t>
         </is>
       </c>
       <c r="B44" s="7" t="inlineStr">
         <is>
-          <t>Feijão — Eng. CDRVIEW Sênior (Alarmística online/API)</t>
+          <t>Rafael — Eng. CDRVIEW Sênior (Parser/Ingestão/Redução/API)</t>
         </is>
       </c>
       <c r="C44" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="D44" s="20">
+        <v>5</v>
+      </c>
+      <c r="D44" s="19">
         <f>C44*0.5</f>
         <v/>
       </c>
-      <c r="E44" s="21" t="n">
+      <c r="E44" s="20" t="n">
         <v>0.4</v>
       </c>
-      <c r="F44" s="17">
-        <f>Papéis!D11</f>
+      <c r="F44" s="16">
+        <f>Papéis!D10</f>
         <v/>
       </c>
       <c r="G44" s="10">
         <f>D44*E44*F44</f>
         <v/>
       </c>
-      <c r="H44" s="16">
-        <f>Papéis!B11</f>
+      <c r="H44" s="15">
+        <f>Papéis!B10</f>
         <v/>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="7" t="inlineStr">
         <is>
-          <t>Fase 5 — Streaming incremental completo (MLOps)</t>
+          <t>Fase 5 — Streaming incremental completo (rede e engajamento)</t>
         </is>
       </c>
       <c r="B45" s="7" t="inlineStr">
         <is>
-          <t>Andréia — QA Sênior</t>
+          <t>Feijão — Eng. CDRVIEW Sênior (Alarmística online/API)</t>
         </is>
       </c>
       <c r="C45" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="D45" s="20">
+        <v>5</v>
+      </c>
+      <c r="D45" s="19">
         <f>C45*0.5</f>
         <v/>
       </c>
-      <c r="E45" s="21" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="F45" s="17">
-        <f>Papéis!D12</f>
+      <c r="E45" s="20" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="F45" s="16">
+        <f>Papéis!D11</f>
         <v/>
       </c>
       <c r="G45" s="10">
         <f>D45*E45*F45</f>
         <v/>
       </c>
-      <c r="H45" s="16">
-        <f>Papéis!B12</f>
+      <c r="H45" s="15">
+        <f>Papéis!B11</f>
         <v/>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="7" t="inlineStr">
         <is>
-          <t>Fase 5 — Streaming incremental completo (MLOps)</t>
+          <t>Fase 5 — Streaming incremental completo (rede e engajamento)</t>
         </is>
       </c>
       <c r="B46" s="7" t="inlineStr">
         <is>
-          <t>CS — Implantação/Rollout</t>
+          <t>Andréia — QA Sênior</t>
         </is>
       </c>
       <c r="C46" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="D46" s="20">
+        <v>5</v>
+      </c>
+      <c r="D46" s="19">
         <f>C46*0.5</f>
         <v/>
       </c>
-      <c r="E46" s="21" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="F46" s="17">
-        <f>Papéis!D13</f>
+      <c r="E46" s="20" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F46" s="16">
+        <f>Papéis!D12</f>
         <v/>
       </c>
       <c r="G46" s="10">
         <f>D46*E46*F46</f>
         <v/>
       </c>
-      <c r="H46" s="16">
+      <c r="H46" s="15">
+        <f>Papéis!B12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="7" t="inlineStr">
+        <is>
+          <t>Fase 5 — Streaming incremental completo (rede e engajamento)</t>
+        </is>
+      </c>
+      <c r="B47" s="7" t="inlineStr">
+        <is>
+          <t>CS — Implantação/Rollout</t>
+        </is>
+      </c>
+      <c r="C47" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="D47" s="19">
+        <f>C47*0.5</f>
+        <v/>
+      </c>
+      <c r="E47" s="20" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F47" s="16">
+        <f>Papéis!D13</f>
+        <v/>
+      </c>
+      <c r="G47" s="10">
+        <f>D47*E47*F47</f>
+        <v/>
+      </c>
+      <c r="H47" s="15">
         <f>Papéis!B13</f>
         <v/>
       </c>
     </row>
-    <row r="47">
-      <c r="A47" s="22" t="inlineStr">
-        <is>
-          <t>Subtotal — Fase 5 — Streaming incremental completo (MLOps)</t>
-        </is>
-      </c>
-      <c r="B47" s="23" t="n"/>
-      <c r="C47" s="23" t="n"/>
-      <c r="D47" s="23" t="n"/>
-      <c r="E47" s="23" t="n"/>
-      <c r="F47" s="23" t="n"/>
-      <c r="G47" s="24">
-        <f>SUM(G38:G46)</f>
-        <v/>
-      </c>
-      <c r="H47" s="23" t="n"/>
-    </row>
-    <row r="49">
-      <c r="A49" s="7" t="inlineStr">
-        <is>
-          <t>Fase 6 — Rollout nacional</t>
-        </is>
-      </c>
-      <c r="B49" s="7" t="inlineStr">
-        <is>
-          <t>PM / Coordenação geral</t>
-        </is>
-      </c>
-      <c r="C49" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="D49" s="20">
-        <f>C49*0.5</f>
-        <v/>
-      </c>
-      <c r="E49" s="21" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="F49" s="17">
-        <f>Papéis!D4</f>
-        <v/>
-      </c>
-      <c r="G49" s="10">
-        <f>D49*E49*F49</f>
-        <v/>
-      </c>
-      <c r="H49" s="16">
-        <f>Papéis!B4</f>
-        <v/>
-      </c>
+    <row r="48">
+      <c r="A48" s="21" t="inlineStr">
+        <is>
+          <t>Subtotal — Fase 5 — Streaming incremental completo (rede e engajamento)</t>
+        </is>
+      </c>
+      <c r="B48" s="22" t="n"/>
+      <c r="C48" s="22" t="n"/>
+      <c r="D48" s="22" t="n"/>
+      <c r="E48" s="22" t="n"/>
+      <c r="F48" s="22" t="n"/>
+      <c r="G48" s="23">
+        <f>SUM(G39:G47)</f>
+        <v/>
+      </c>
+      <c r="H48" s="22" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="7" t="inlineStr">
@@ -2665,29 +2670,29 @@
       </c>
       <c r="B50" s="7" t="inlineStr">
         <is>
-          <t>Engenheiro de Dados Sênior — Pipelines/Tensores</t>
+          <t>PM / Coordenação geral</t>
         </is>
       </c>
       <c r="C50" s="7" t="n">
         <v>6</v>
       </c>
-      <c r="D50" s="20">
+      <c r="D50" s="19">
         <f>C50*0.5</f>
         <v/>
       </c>
-      <c r="E50" s="21" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="F50" s="17">
-        <f>Papéis!D6</f>
+      <c r="E50" s="20" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="F50" s="16">
+        <f>Papéis!D4</f>
         <v/>
       </c>
       <c r="G50" s="10">
         <f>D50*E50*F50</f>
         <v/>
       </c>
-      <c r="H50" s="19">
-        <f>Papéis!B6</f>
+      <c r="H50" s="15">
+        <f>Papéis!B4</f>
         <v/>
       </c>
     </row>
@@ -2699,29 +2704,29 @@
       </c>
       <c r="B51" s="7" t="inlineStr">
         <is>
-          <t>Engenheiro de Software Sênior — Dashboards/API</t>
+          <t>Engenheiro de Dados Sênior — Pipelines/Tensores</t>
         </is>
       </c>
       <c r="C51" s="7" t="n">
         <v>6</v>
       </c>
-      <c r="D51" s="20">
+      <c r="D51" s="19">
         <f>C51*0.5</f>
         <v/>
       </c>
-      <c r="E51" s="21" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="F51" s="17">
-        <f>Papéis!D8</f>
+      <c r="E51" s="20" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F51" s="16">
+        <f>Papéis!D6</f>
         <v/>
       </c>
       <c r="G51" s="10">
         <f>D51*E51*F51</f>
         <v/>
       </c>
-      <c r="H51" s="19">
-        <f>Papéis!B8</f>
+      <c r="H51" s="18">
+        <f>Papéis!B6</f>
         <v/>
       </c>
     </row>
@@ -2733,29 +2738,29 @@
       </c>
       <c r="B52" s="7" t="inlineStr">
         <is>
-          <t>Rafael — Eng. CDRVIEW Sênior (Parser/Ingestão/Redução/API)</t>
+          <t>Engenheiro de Software Sênior — Dashboards/API</t>
         </is>
       </c>
       <c r="C52" s="7" t="n">
         <v>6</v>
       </c>
-      <c r="D52" s="20">
+      <c r="D52" s="19">
         <f>C52*0.5</f>
         <v/>
       </c>
-      <c r="E52" s="21" t="n">
+      <c r="E52" s="20" t="n">
         <v>0.2</v>
       </c>
-      <c r="F52" s="17">
-        <f>Papéis!D10</f>
+      <c r="F52" s="16">
+        <f>Papéis!D8</f>
         <v/>
       </c>
       <c r="G52" s="10">
         <f>D52*E52*F52</f>
         <v/>
       </c>
-      <c r="H52" s="16">
-        <f>Papéis!B10</f>
+      <c r="H52" s="18">
+        <f>Papéis!B8</f>
         <v/>
       </c>
     </row>
@@ -2767,29 +2772,29 @@
       </c>
       <c r="B53" s="7" t="inlineStr">
         <is>
-          <t>Feijão — Eng. CDRVIEW Sênior (Alarmística online/API)</t>
+          <t>Rafael — Eng. CDRVIEW Sênior (Parser/Ingestão/Redução/API)</t>
         </is>
       </c>
       <c r="C53" s="7" t="n">
         <v>6</v>
       </c>
-      <c r="D53" s="20">
+      <c r="D53" s="19">
         <f>C53*0.5</f>
         <v/>
       </c>
-      <c r="E53" s="21" t="n">
+      <c r="E53" s="20" t="n">
         <v>0.2</v>
       </c>
-      <c r="F53" s="17">
-        <f>Papéis!D11</f>
+      <c r="F53" s="16">
+        <f>Papéis!D10</f>
         <v/>
       </c>
       <c r="G53" s="10">
         <f>D53*E53*F53</f>
         <v/>
       </c>
-      <c r="H53" s="16">
-        <f>Papéis!B11</f>
+      <c r="H53" s="15">
+        <f>Papéis!B10</f>
         <v/>
       </c>
     </row>
@@ -2801,29 +2806,29 @@
       </c>
       <c r="B54" s="7" t="inlineStr">
         <is>
-          <t>Andréia — QA Sênior</t>
+          <t>Feijão — Eng. CDRVIEW Sênior (Alarmística online/API)</t>
         </is>
       </c>
       <c r="C54" s="7" t="n">
         <v>6</v>
       </c>
-      <c r="D54" s="20">
+      <c r="D54" s="19">
         <f>C54*0.5</f>
         <v/>
       </c>
-      <c r="E54" s="21" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="F54" s="17">
-        <f>Papéis!D12</f>
+      <c r="E54" s="20" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F54" s="16">
+        <f>Papéis!D11</f>
         <v/>
       </c>
       <c r="G54" s="10">
         <f>D54*E54*F54</f>
         <v/>
       </c>
-      <c r="H54" s="16">
-        <f>Papéis!B12</f>
+      <c r="H54" s="15">
+        <f>Papéis!B11</f>
         <v/>
       </c>
     </row>
@@ -2835,76 +2840,110 @@
       </c>
       <c r="B55" s="7" t="inlineStr">
         <is>
-          <t>CS — Implantação/Rollout</t>
+          <t>Andréia — QA Sênior</t>
         </is>
       </c>
       <c r="C55" s="7" t="n">
         <v>6</v>
       </c>
-      <c r="D55" s="20">
+      <c r="D55" s="19">
         <f>C55*0.5</f>
         <v/>
       </c>
-      <c r="E55" s="21" t="n">
-        <v>1</v>
-      </c>
-      <c r="F55" s="17">
-        <f>Papéis!D13</f>
+      <c r="E55" s="20" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="F55" s="16">
+        <f>Papéis!D12</f>
         <v/>
       </c>
       <c r="G55" s="10">
         <f>D55*E55*F55</f>
         <v/>
       </c>
-      <c r="H55" s="16">
+      <c r="H55" s="15">
+        <f>Papéis!B12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="7" t="inlineStr">
+        <is>
+          <t>Fase 6 — Rollout nacional</t>
+        </is>
+      </c>
+      <c r="B56" s="7" t="inlineStr">
+        <is>
+          <t>CS — Implantação/Rollout</t>
+        </is>
+      </c>
+      <c r="C56" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="D56" s="19">
+        <f>C56*0.5</f>
+        <v/>
+      </c>
+      <c r="E56" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="F56" s="16">
+        <f>Papéis!D13</f>
+        <v/>
+      </c>
+      <c r="G56" s="10">
+        <f>D56*E56*F56</f>
+        <v/>
+      </c>
+      <c r="H56" s="15">
         <f>Papéis!B13</f>
         <v/>
       </c>
     </row>
-    <row r="56">
-      <c r="A56" s="22" t="inlineStr">
+    <row r="57">
+      <c r="A57" s="21" t="inlineStr">
         <is>
           <t>Subtotal — Fase 6 — Rollout nacional</t>
         </is>
       </c>
-      <c r="B56" s="23" t="n"/>
-      <c r="C56" s="23" t="n"/>
-      <c r="D56" s="23" t="n"/>
-      <c r="E56" s="23" t="n"/>
-      <c r="F56" s="23" t="n"/>
-      <c r="G56" s="24">
-        <f>SUM(G49:G55)</f>
-        <v/>
-      </c>
-      <c r="H56" s="23" t="n"/>
-    </row>
-    <row r="58">
-      <c r="A58" s="12" t="inlineStr">
+      <c r="B57" s="22" t="n"/>
+      <c r="C57" s="22" t="n"/>
+      <c r="D57" s="22" t="n"/>
+      <c r="E57" s="22" t="n"/>
+      <c r="F57" s="22" t="n"/>
+      <c r="G57" s="23">
+        <f>SUM(G50:G56)</f>
+        <v/>
+      </c>
+      <c r="H57" s="22" t="n"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="11" t="inlineStr">
         <is>
           <t>CUSTO TOTAL DO PROJETO</t>
         </is>
       </c>
-      <c r="B58" s="12" t="n"/>
-      <c r="C58" s="12" t="n"/>
-      <c r="D58" s="12" t="n"/>
-      <c r="E58" s="12" t="n"/>
-      <c r="F58" s="12" t="n"/>
-      <c r="G58" s="13">
-        <f>G12+G18+G26+G36+G47+G56</f>
-        <v/>
-      </c>
-      <c r="H58" s="12" t="n"/>
+      <c r="B59" s="11" t="n"/>
+      <c r="C59" s="11" t="n"/>
+      <c r="D59" s="11" t="n"/>
+      <c r="E59" s="11" t="n"/>
+      <c r="F59" s="11" t="n"/>
+      <c r="G59" s="12">
+        <f>G13+G19+G27+G37+G48+G57</f>
+        <v/>
+      </c>
+      <c r="H59" s="11" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="8">
-    <mergeCell ref="A47:F47"/>
-    <mergeCell ref="A36:F36"/>
-    <mergeCell ref="A58:F58"/>
-    <mergeCell ref="A12:F12"/>
-    <mergeCell ref="A18:F18"/>
+    <mergeCell ref="A13:F13"/>
+    <mergeCell ref="A19:F19"/>
+    <mergeCell ref="A37:F37"/>
+    <mergeCell ref="A27:F27"/>
     <mergeCell ref="A1:H1"/>
-    <mergeCell ref="A26:F26"/>
-    <mergeCell ref="A56:F56"/>
+    <mergeCell ref="A48:F48"/>
+    <mergeCell ref="A59:F59"/>
+    <mergeCell ref="A57:F57"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3112,247 +3151,247 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="25" t="inlineStr">
+      <c r="A4" s="24" t="inlineStr">
         <is>
           <t>Fase 1 — Personas &amp; Qualidade de Deslocamento</t>
         </is>
       </c>
-      <c r="B4" s="25" t="inlineStr">
+      <c r="B4" s="24" t="inlineStr">
         <is>
           <t>Sprint 1</t>
         </is>
       </c>
-      <c r="C4" s="25" t="inlineStr">
-        <is>
-          <t>Sprint 4</t>
-        </is>
-      </c>
-      <c r="D4" s="26" t="n"/>
-      <c r="E4" s="26" t="n"/>
-      <c r="F4" s="26" t="n"/>
-      <c r="G4" s="26" t="n"/>
-      <c r="H4" s="27" t="n"/>
-      <c r="I4" s="27" t="n"/>
-      <c r="J4" s="27" t="n"/>
-      <c r="K4" s="27" t="n"/>
-      <c r="L4" s="27" t="n"/>
-      <c r="M4" s="27" t="n"/>
-      <c r="N4" s="27" t="n"/>
-      <c r="O4" s="27" t="n"/>
-      <c r="P4" s="27" t="n"/>
-      <c r="Q4" s="27" t="n"/>
-      <c r="R4" s="27" t="n"/>
-      <c r="S4" s="27" t="n"/>
-      <c r="T4" s="27" t="n"/>
-      <c r="U4" s="27" t="n"/>
-      <c r="V4" s="27" t="n"/>
-      <c r="W4" s="27" t="n"/>
-      <c r="X4" s="27" t="n"/>
-      <c r="Y4" s="27" t="n"/>
-      <c r="Z4" s="27" t="n"/>
+      <c r="C4" s="24" t="inlineStr">
+        <is>
+          <t>Sprint 5</t>
+        </is>
+      </c>
+      <c r="D4" s="25" t="n"/>
+      <c r="E4" s="25" t="n"/>
+      <c r="F4" s="25" t="n"/>
+      <c r="G4" s="25" t="n"/>
+      <c r="H4" s="25" t="n"/>
+      <c r="I4" s="26" t="n"/>
+      <c r="J4" s="26" t="n"/>
+      <c r="K4" s="26" t="n"/>
+      <c r="L4" s="26" t="n"/>
+      <c r="M4" s="26" t="n"/>
+      <c r="N4" s="26" t="n"/>
+      <c r="O4" s="26" t="n"/>
+      <c r="P4" s="26" t="n"/>
+      <c r="Q4" s="26" t="n"/>
+      <c r="R4" s="26" t="n"/>
+      <c r="S4" s="26" t="n"/>
+      <c r="T4" s="26" t="n"/>
+      <c r="U4" s="26" t="n"/>
+      <c r="V4" s="26" t="n"/>
+      <c r="W4" s="26" t="n"/>
+      <c r="X4" s="26" t="n"/>
+      <c r="Y4" s="26" t="n"/>
+      <c r="Z4" s="26" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="25" t="inlineStr">
+      <c r="A5" s="24" t="inlineStr">
         <is>
           <t>Fase 2 — Dashboard da Alarmística existente</t>
         </is>
       </c>
-      <c r="B5" s="25" t="inlineStr">
+      <c r="B5" s="24" t="inlineStr">
         <is>
           <t>Sprint 1</t>
         </is>
       </c>
-      <c r="C5" s="25" t="inlineStr">
+      <c r="C5" s="24" t="inlineStr">
         <is>
           <t>Sprint 2</t>
         </is>
       </c>
-      <c r="D5" s="28" t="n"/>
-      <c r="E5" s="28" t="n"/>
-      <c r="F5" s="27" t="n"/>
-      <c r="G5" s="27" t="n"/>
-      <c r="H5" s="27" t="n"/>
-      <c r="I5" s="27" t="n"/>
-      <c r="J5" s="27" t="n"/>
-      <c r="K5" s="27" t="n"/>
-      <c r="L5" s="27" t="n"/>
-      <c r="M5" s="27" t="n"/>
-      <c r="N5" s="27" t="n"/>
-      <c r="O5" s="27" t="n"/>
-      <c r="P5" s="27" t="n"/>
-      <c r="Q5" s="27" t="n"/>
-      <c r="R5" s="27" t="n"/>
-      <c r="S5" s="27" t="n"/>
-      <c r="T5" s="27" t="n"/>
-      <c r="U5" s="27" t="n"/>
-      <c r="V5" s="27" t="n"/>
-      <c r="W5" s="27" t="n"/>
-      <c r="X5" s="27" t="n"/>
-      <c r="Y5" s="27" t="n"/>
-      <c r="Z5" s="27" t="n"/>
+      <c r="D5" s="27" t="n"/>
+      <c r="E5" s="27" t="n"/>
+      <c r="F5" s="26" t="n"/>
+      <c r="G5" s="26" t="n"/>
+      <c r="H5" s="26" t="n"/>
+      <c r="I5" s="26" t="n"/>
+      <c r="J5" s="26" t="n"/>
+      <c r="K5" s="26" t="n"/>
+      <c r="L5" s="26" t="n"/>
+      <c r="M5" s="26" t="n"/>
+      <c r="N5" s="26" t="n"/>
+      <c r="O5" s="26" t="n"/>
+      <c r="P5" s="26" t="n"/>
+      <c r="Q5" s="26" t="n"/>
+      <c r="R5" s="26" t="n"/>
+      <c r="S5" s="26" t="n"/>
+      <c r="T5" s="26" t="n"/>
+      <c r="U5" s="26" t="n"/>
+      <c r="V5" s="26" t="n"/>
+      <c r="W5" s="26" t="n"/>
+      <c r="X5" s="26" t="n"/>
+      <c r="Y5" s="26" t="n"/>
+      <c r="Z5" s="26" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="25" t="inlineStr">
+      <c r="A6" s="24" t="inlineStr">
         <is>
           <t>Fase 3 — Analytics novo sobre a Alarmística</t>
         </is>
       </c>
-      <c r="B6" s="25" t="inlineStr">
-        <is>
-          <t>Sprint 5</t>
-        </is>
-      </c>
-      <c r="C6" s="25" t="inlineStr">
-        <is>
-          <t>Sprint 7</t>
-        </is>
-      </c>
-      <c r="D6" s="27" t="n"/>
-      <c r="E6" s="27" t="n"/>
-      <c r="F6" s="27" t="n"/>
-      <c r="G6" s="27" t="n"/>
-      <c r="H6" s="29" t="n"/>
-      <c r="I6" s="29" t="n"/>
-      <c r="J6" s="29" t="n"/>
-      <c r="K6" s="27" t="n"/>
-      <c r="L6" s="27" t="n"/>
-      <c r="M6" s="27" t="n"/>
-      <c r="N6" s="27" t="n"/>
-      <c r="O6" s="27" t="n"/>
-      <c r="P6" s="27" t="n"/>
-      <c r="Q6" s="27" t="n"/>
-      <c r="R6" s="27" t="n"/>
-      <c r="S6" s="27" t="n"/>
-      <c r="T6" s="27" t="n"/>
-      <c r="U6" s="27" t="n"/>
-      <c r="V6" s="27" t="n"/>
-      <c r="W6" s="27" t="n"/>
-      <c r="X6" s="27" t="n"/>
-      <c r="Y6" s="27" t="n"/>
-      <c r="Z6" s="27" t="n"/>
+      <c r="B6" s="24" t="inlineStr">
+        <is>
+          <t>Sprint 6</t>
+        </is>
+      </c>
+      <c r="C6" s="24" t="inlineStr">
+        <is>
+          <t>Sprint 8</t>
+        </is>
+      </c>
+      <c r="D6" s="26" t="n"/>
+      <c r="E6" s="26" t="n"/>
+      <c r="F6" s="26" t="n"/>
+      <c r="G6" s="26" t="n"/>
+      <c r="H6" s="26" t="n"/>
+      <c r="I6" s="28" t="n"/>
+      <c r="J6" s="28" t="n"/>
+      <c r="K6" s="28" t="n"/>
+      <c r="L6" s="26" t="n"/>
+      <c r="M6" s="26" t="n"/>
+      <c r="N6" s="26" t="n"/>
+      <c r="O6" s="26" t="n"/>
+      <c r="P6" s="26" t="n"/>
+      <c r="Q6" s="26" t="n"/>
+      <c r="R6" s="26" t="n"/>
+      <c r="S6" s="26" t="n"/>
+      <c r="T6" s="26" t="n"/>
+      <c r="U6" s="26" t="n"/>
+      <c r="V6" s="26" t="n"/>
+      <c r="W6" s="26" t="n"/>
+      <c r="X6" s="26" t="n"/>
+      <c r="Y6" s="26" t="n"/>
+      <c r="Z6" s="26" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="25" t="inlineStr">
+      <c r="A7" s="24" t="inlineStr">
         <is>
           <t>Fase 4 — Topologia de rede + Priorização de alertas</t>
         </is>
       </c>
-      <c r="B7" s="25" t="inlineStr">
-        <is>
-          <t>Sprint 8</t>
-        </is>
-      </c>
-      <c r="C7" s="25" t="inlineStr">
-        <is>
-          <t>Sprint 11</t>
-        </is>
-      </c>
-      <c r="D7" s="27" t="n"/>
-      <c r="E7" s="27" t="n"/>
-      <c r="F7" s="27" t="n"/>
-      <c r="G7" s="27" t="n"/>
-      <c r="H7" s="27" t="n"/>
-      <c r="I7" s="27" t="n"/>
-      <c r="J7" s="27" t="n"/>
-      <c r="K7" s="30" t="n"/>
-      <c r="L7" s="30" t="n"/>
-      <c r="M7" s="30" t="n"/>
-      <c r="N7" s="30" t="n"/>
-      <c r="O7" s="27" t="n"/>
-      <c r="P7" s="27" t="n"/>
-      <c r="Q7" s="27" t="n"/>
-      <c r="R7" s="27" t="n"/>
-      <c r="S7" s="27" t="n"/>
-      <c r="T7" s="27" t="n"/>
-      <c r="U7" s="27" t="n"/>
-      <c r="V7" s="27" t="n"/>
-      <c r="W7" s="27" t="n"/>
-      <c r="X7" s="27" t="n"/>
-      <c r="Y7" s="27" t="n"/>
-      <c r="Z7" s="27" t="n"/>
+      <c r="B7" s="24" t="inlineStr">
+        <is>
+          <t>Sprint 9</t>
+        </is>
+      </c>
+      <c r="C7" s="24" t="inlineStr">
+        <is>
+          <t>Sprint 12</t>
+        </is>
+      </c>
+      <c r="D7" s="26" t="n"/>
+      <c r="E7" s="26" t="n"/>
+      <c r="F7" s="26" t="n"/>
+      <c r="G7" s="26" t="n"/>
+      <c r="H7" s="26" t="n"/>
+      <c r="I7" s="26" t="n"/>
+      <c r="J7" s="26" t="n"/>
+      <c r="K7" s="26" t="n"/>
+      <c r="L7" s="29" t="n"/>
+      <c r="M7" s="29" t="n"/>
+      <c r="N7" s="29" t="n"/>
+      <c r="O7" s="29" t="n"/>
+      <c r="P7" s="26" t="n"/>
+      <c r="Q7" s="26" t="n"/>
+      <c r="R7" s="26" t="n"/>
+      <c r="S7" s="26" t="n"/>
+      <c r="T7" s="26" t="n"/>
+      <c r="U7" s="26" t="n"/>
+      <c r="V7" s="26" t="n"/>
+      <c r="W7" s="26" t="n"/>
+      <c r="X7" s="26" t="n"/>
+      <c r="Y7" s="26" t="n"/>
+      <c r="Z7" s="26" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="25" t="inlineStr">
-        <is>
-          <t>Fase 5 — Streaming incremental completo (MLOps)</t>
-        </is>
-      </c>
-      <c r="B8" s="25" t="inlineStr">
-        <is>
-          <t>Sprint 12</t>
-        </is>
-      </c>
-      <c r="C8" s="25" t="inlineStr">
+      <c r="A8" s="24" t="inlineStr">
+        <is>
+          <t>Fase 5 — Streaming incremental completo (rede e engajamento)</t>
+        </is>
+      </c>
+      <c r="B8" s="24" t="inlineStr">
+        <is>
+          <t>Sprint 13</t>
+        </is>
+      </c>
+      <c r="C8" s="24" t="inlineStr">
         <is>
           <t>Sprint 17</t>
         </is>
       </c>
-      <c r="D8" s="27" t="n"/>
-      <c r="E8" s="27" t="n"/>
-      <c r="F8" s="27" t="n"/>
-      <c r="G8" s="27" t="n"/>
-      <c r="H8" s="27" t="n"/>
-      <c r="I8" s="27" t="n"/>
-      <c r="J8" s="27" t="n"/>
-      <c r="K8" s="27" t="n"/>
-      <c r="L8" s="27" t="n"/>
-      <c r="M8" s="27" t="n"/>
-      <c r="N8" s="27" t="n"/>
-      <c r="O8" s="31" t="n"/>
-      <c r="P8" s="31" t="n"/>
-      <c r="Q8" s="31" t="n"/>
-      <c r="R8" s="31" t="n"/>
-      <c r="S8" s="31" t="n"/>
-      <c r="T8" s="31" t="n"/>
-      <c r="U8" s="27" t="n"/>
-      <c r="V8" s="27" t="n"/>
-      <c r="W8" s="27" t="n"/>
-      <c r="X8" s="27" t="n"/>
-      <c r="Y8" s="27" t="n"/>
-      <c r="Z8" s="27" t="n"/>
+      <c r="D8" s="26" t="n"/>
+      <c r="E8" s="26" t="n"/>
+      <c r="F8" s="26" t="n"/>
+      <c r="G8" s="26" t="n"/>
+      <c r="H8" s="26" t="n"/>
+      <c r="I8" s="26" t="n"/>
+      <c r="J8" s="26" t="n"/>
+      <c r="K8" s="26" t="n"/>
+      <c r="L8" s="26" t="n"/>
+      <c r="M8" s="26" t="n"/>
+      <c r="N8" s="26" t="n"/>
+      <c r="O8" s="26" t="n"/>
+      <c r="P8" s="30" t="n"/>
+      <c r="Q8" s="30" t="n"/>
+      <c r="R8" s="30" t="n"/>
+      <c r="S8" s="30" t="n"/>
+      <c r="T8" s="30" t="n"/>
+      <c r="U8" s="26" t="n"/>
+      <c r="V8" s="26" t="n"/>
+      <c r="W8" s="26" t="n"/>
+      <c r="X8" s="26" t="n"/>
+      <c r="Y8" s="26" t="n"/>
+      <c r="Z8" s="26" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="25" t="inlineStr">
+      <c r="A9" s="24" t="inlineStr">
         <is>
           <t>Fase 6 — Rollout nacional</t>
         </is>
       </c>
-      <c r="B9" s="25" t="inlineStr">
+      <c r="B9" s="24" t="inlineStr">
         <is>
           <t>Sprint 18</t>
         </is>
       </c>
-      <c r="C9" s="25" t="inlineStr">
+      <c r="C9" s="24" t="inlineStr">
         <is>
           <t>Sprint 23</t>
         </is>
       </c>
-      <c r="D9" s="27" t="n"/>
-      <c r="E9" s="27" t="n"/>
-      <c r="F9" s="27" t="n"/>
-      <c r="G9" s="27" t="n"/>
-      <c r="H9" s="27" t="n"/>
-      <c r="I9" s="27" t="n"/>
-      <c r="J9" s="27" t="n"/>
-      <c r="K9" s="27" t="n"/>
-      <c r="L9" s="27" t="n"/>
-      <c r="M9" s="27" t="n"/>
-      <c r="N9" s="27" t="n"/>
-      <c r="O9" s="27" t="n"/>
-      <c r="P9" s="27" t="n"/>
-      <c r="Q9" s="27" t="n"/>
-      <c r="R9" s="27" t="n"/>
-      <c r="S9" s="27" t="n"/>
-      <c r="T9" s="27" t="n"/>
-      <c r="U9" s="32" t="n"/>
-      <c r="V9" s="32" t="n"/>
-      <c r="W9" s="32" t="n"/>
-      <c r="X9" s="32" t="n"/>
-      <c r="Y9" s="32" t="n"/>
-      <c r="Z9" s="32" t="n"/>
+      <c r="D9" s="26" t="n"/>
+      <c r="E9" s="26" t="n"/>
+      <c r="F9" s="26" t="n"/>
+      <c r="G9" s="26" t="n"/>
+      <c r="H9" s="26" t="n"/>
+      <c r="I9" s="26" t="n"/>
+      <c r="J9" s="26" t="n"/>
+      <c r="K9" s="26" t="n"/>
+      <c r="L9" s="26" t="n"/>
+      <c r="M9" s="26" t="n"/>
+      <c r="N9" s="26" t="n"/>
+      <c r="O9" s="26" t="n"/>
+      <c r="P9" s="26" t="n"/>
+      <c r="Q9" s="26" t="n"/>
+      <c r="R9" s="26" t="n"/>
+      <c r="S9" s="26" t="n"/>
+      <c r="T9" s="26" t="n"/>
+      <c r="U9" s="31" t="n"/>
+      <c r="V9" s="31" t="n"/>
+      <c r="W9" s="31" t="n"/>
+      <c r="X9" s="31" t="n"/>
+      <c r="Y9" s="31" t="n"/>
+      <c r="Z9" s="31" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="33" t="inlineStr">
+      <c r="A11" s="32" t="inlineStr">
         <is>
           <t>Cronograma sequencial-enxuto (1 pessoa por papel). Compressão possível adicionando FTE — ver Resumo Executivo.</t>
         </is>
@@ -3448,27 +3487,27 @@
           <t>PM / Coordenação geral</t>
         </is>
       </c>
-      <c r="B4" s="16" t="inlineStr">
+      <c r="B4" s="15" t="inlineStr">
         <is>
           <t>Vísent</t>
         </is>
       </c>
-      <c r="C4" s="34" t="n">
+      <c r="C4" s="33" t="n">
         <v>0.5</v>
       </c>
-      <c r="D4" s="35" t="n">
+      <c r="D4" s="34" t="n">
         <v>0.3</v>
       </c>
-      <c r="E4" s="35" t="n">
+      <c r="E4" s="34" t="n">
         <v>0.3</v>
       </c>
-      <c r="F4" s="34" t="n">
+      <c r="F4" s="33" t="n">
         <v>0.4</v>
       </c>
-      <c r="G4" s="34" t="n">
+      <c r="G4" s="33" t="n">
         <v>0.5</v>
       </c>
-      <c r="H4" s="34" t="n">
+      <c r="H4" s="33" t="n">
         <v>0.4</v>
       </c>
     </row>
@@ -3478,25 +3517,25 @@
           <t>Arquiteto de Dados/Soluções Sênior</t>
         </is>
       </c>
-      <c r="B5" s="19" t="inlineStr">
+      <c r="B5" s="18" t="inlineStr">
         <is>
           <t>Brintell</t>
         </is>
       </c>
-      <c r="C5" s="34" t="n">
+      <c r="C5" s="33" t="n">
         <v>0.5</v>
       </c>
-      <c r="D5" s="36" t="n"/>
-      <c r="E5" s="35" t="n">
+      <c r="D5" s="35" t="n"/>
+      <c r="E5" s="34" t="n">
         <v>0.1</v>
       </c>
-      <c r="F5" s="35" t="n">
+      <c r="F5" s="34" t="n">
         <v>0.3</v>
       </c>
-      <c r="G5" s="34" t="n">
+      <c r="G5" s="33" t="n">
         <v>0.5</v>
       </c>
-      <c r="H5" s="36" t="n"/>
+      <c r="H5" s="35" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
@@ -3504,21 +3543,21 @@
           <t>Engenheiro de Dados Sênior — Pipelines/Tensores</t>
         </is>
       </c>
-      <c r="B6" s="19" t="inlineStr">
+      <c r="B6" s="18" t="inlineStr">
         <is>
           <t>Brintell</t>
         </is>
       </c>
-      <c r="C6" s="37" t="n">
+      <c r="C6" s="36" t="n">
         <v>1</v>
       </c>
-      <c r="D6" s="36" t="n"/>
-      <c r="E6" s="36" t="n"/>
-      <c r="F6" s="37" t="n">
+      <c r="D6" s="35" t="n"/>
+      <c r="E6" s="35" t="n"/>
+      <c r="F6" s="36" t="n">
         <v>0.8</v>
       </c>
-      <c r="G6" s="36" t="n"/>
-      <c r="H6" s="35" t="n">
+      <c r="G6" s="35" t="n"/>
+      <c r="H6" s="34" t="n">
         <v>0.3</v>
       </c>
     </row>
@@ -3528,25 +3567,25 @@
           <t>Cientista de Dados Sênior — ML/Personas/Markov/Bayes</t>
         </is>
       </c>
-      <c r="B7" s="19" t="inlineStr">
+      <c r="B7" s="18" t="inlineStr">
         <is>
           <t>Brintell</t>
         </is>
       </c>
-      <c r="C7" s="37" t="n">
+      <c r="C7" s="36" t="n">
         <v>1</v>
       </c>
-      <c r="D7" s="36" t="n"/>
-      <c r="E7" s="37" t="n">
+      <c r="D7" s="35" t="n"/>
+      <c r="E7" s="36" t="n">
         <v>1</v>
       </c>
-      <c r="F7" s="34" t="n">
+      <c r="F7" s="33" t="n">
         <v>0.6</v>
       </c>
-      <c r="G7" s="34" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="H7" s="36" t="n"/>
+      <c r="G7" s="33" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="H7" s="35" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="7" t="inlineStr">
@@ -3554,27 +3593,27 @@
           <t>Engenheiro de Software Sênior — Dashboards/API</t>
         </is>
       </c>
-      <c r="B8" s="19" t="inlineStr">
+      <c r="B8" s="18" t="inlineStr">
         <is>
           <t>Brintell</t>
         </is>
       </c>
-      <c r="C8" s="34" t="n">
+      <c r="C8" s="33" t="n">
         <v>0.5</v>
       </c>
-      <c r="D8" s="37" t="n">
+      <c r="D8" s="36" t="n">
         <v>1</v>
       </c>
-      <c r="E8" s="34" t="n">
+      <c r="E8" s="33" t="n">
         <v>0.5</v>
       </c>
-      <c r="F8" s="34" t="n">
+      <c r="F8" s="33" t="n">
         <v>0.6</v>
       </c>
-      <c r="G8" s="34" t="n">
+      <c r="G8" s="33" t="n">
         <v>0.5</v>
       </c>
-      <c r="H8" s="35" t="n">
+      <c r="H8" s="34" t="n">
         <v>0.2</v>
       </c>
     </row>
@@ -3584,19 +3623,21 @@
           <t>Engenheiro de Dados Sênior — MLOps/Streaming</t>
         </is>
       </c>
-      <c r="B9" s="19" t="inlineStr">
+      <c r="B9" s="18" t="inlineStr">
         <is>
           <t>Brintell</t>
         </is>
       </c>
-      <c r="C9" s="36" t="n"/>
-      <c r="D9" s="36" t="n"/>
-      <c r="E9" s="36" t="n"/>
-      <c r="F9" s="36" t="n"/>
-      <c r="G9" s="37" t="n">
-        <v>1</v>
-      </c>
-      <c r="H9" s="36" t="n"/>
+      <c r="C9" s="34" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="D9" s="35" t="n"/>
+      <c r="E9" s="35" t="n"/>
+      <c r="F9" s="35" t="n"/>
+      <c r="G9" s="36" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="H9" s="35" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
@@ -3604,23 +3645,23 @@
           <t>Rafael — Eng. CDRVIEW Sênior (Parser/Ingestão/Redução/API)</t>
         </is>
       </c>
-      <c r="B10" s="16" t="inlineStr">
+      <c r="B10" s="15" t="inlineStr">
         <is>
           <t>Claro/CDRVIEW</t>
         </is>
       </c>
-      <c r="C10" s="35" t="n">
+      <c r="C10" s="34" t="n">
         <v>0.2</v>
       </c>
-      <c r="D10" s="36" t="n"/>
-      <c r="E10" s="36" t="n"/>
-      <c r="F10" s="35" t="n">
+      <c r="D10" s="35" t="n"/>
+      <c r="E10" s="35" t="n"/>
+      <c r="F10" s="34" t="n">
         <v>0.3</v>
       </c>
-      <c r="G10" s="34" t="n">
+      <c r="G10" s="33" t="n">
         <v>0.4</v>
       </c>
-      <c r="H10" s="35" t="n">
+      <c r="H10" s="34" t="n">
         <v>0.2</v>
       </c>
     </row>
@@ -3630,23 +3671,23 @@
           <t>Feijão — Eng. CDRVIEW Sênior (Alarmística online/API)</t>
         </is>
       </c>
-      <c r="B11" s="16" t="inlineStr">
+      <c r="B11" s="15" t="inlineStr">
         <is>
           <t>Claro/CDRVIEW</t>
         </is>
       </c>
-      <c r="C11" s="36" t="n"/>
-      <c r="D11" s="35" t="n">
+      <c r="C11" s="35" t="n"/>
+      <c r="D11" s="34" t="n">
         <v>0.3</v>
       </c>
-      <c r="E11" s="35" t="n">
+      <c r="E11" s="34" t="n">
         <v>0.3</v>
       </c>
-      <c r="F11" s="36" t="n"/>
-      <c r="G11" s="34" t="n">
+      <c r="F11" s="35" t="n"/>
+      <c r="G11" s="33" t="n">
         <v>0.4</v>
       </c>
-      <c r="H11" s="35" t="n">
+      <c r="H11" s="34" t="n">
         <v>0.2</v>
       </c>
     </row>
@@ -3656,27 +3697,27 @@
           <t>Andréia — QA Sênior</t>
         </is>
       </c>
-      <c r="B12" s="16" t="inlineStr">
+      <c r="B12" s="15" t="inlineStr">
         <is>
           <t>Claro/CDRVIEW</t>
         </is>
       </c>
-      <c r="C12" s="35" t="n">
+      <c r="C12" s="34" t="n">
         <v>0.3</v>
       </c>
-      <c r="D12" s="35" t="n">
+      <c r="D12" s="34" t="n">
         <v>0.3</v>
       </c>
-      <c r="E12" s="35" t="n">
+      <c r="E12" s="34" t="n">
         <v>0.3</v>
       </c>
-      <c r="F12" s="34" t="n">
+      <c r="F12" s="33" t="n">
         <v>0.4</v>
       </c>
-      <c r="G12" s="34" t="n">
+      <c r="G12" s="33" t="n">
         <v>0.5</v>
       </c>
-      <c r="H12" s="34" t="n">
+      <c r="H12" s="33" t="n">
         <v>0.4</v>
       </c>
     </row>
@@ -3686,28 +3727,28 @@
           <t>CS — Implantação/Rollout</t>
         </is>
       </c>
-      <c r="B13" s="16" t="inlineStr">
+      <c r="B13" s="15" t="inlineStr">
         <is>
           <t>Claro</t>
         </is>
       </c>
-      <c r="C13" s="35" t="n">
+      <c r="C13" s="34" t="n">
         <v>0.1</v>
       </c>
-      <c r="D13" s="36" t="n"/>
-      <c r="E13" s="36" t="n"/>
-      <c r="F13" s="35" t="n">
+      <c r="D13" s="35" t="n"/>
+      <c r="E13" s="35" t="n"/>
+      <c r="F13" s="34" t="n">
         <v>0.2</v>
       </c>
-      <c r="G13" s="35" t="n">
+      <c r="G13" s="34" t="n">
         <v>0.2</v>
       </c>
-      <c r="H13" s="37" t="n">
+      <c r="H13" s="36" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="33" t="inlineStr">
+      <c r="A15" s="32" t="inlineStr">
         <is>
           <t>Vermelho = alocação alta (≥80%) · Amarelo = média (40–79%) · Verde = pontual (&lt;40%)</t>
         </is>
@@ -3789,16 +3830,16 @@
           <t>PM / Coordenação geral</t>
         </is>
       </c>
-      <c r="B4" s="16" t="inlineStr">
+      <c r="B4" s="15" t="inlineStr">
         <is>
           <t>Vísent</t>
         </is>
       </c>
-      <c r="C4" s="17">
+      <c r="C4" s="16">
         <f>Papéis!D4</f>
         <v/>
       </c>
-      <c r="D4" s="20">
+      <c r="D4" s="19">
         <f>SUMPRODUCT(('Custo Detalhado'!$B$4:$B$200=A4)*'Custo Detalhado'!$D$4:$D$200*'Custo Detalhado'!$E$4:$E$200)</f>
         <v/>
       </c>
@@ -3806,7 +3847,7 @@
         <f>SUMIF('Custo Detalhado'!B:B,A4,'Custo Detalhado'!G:G)</f>
         <v/>
       </c>
-      <c r="F4" s="21">
+      <c r="F4" s="20">
         <f>E4/E14</f>
         <v/>
       </c>
@@ -3817,16 +3858,16 @@
           <t>Arquiteto de Dados/Soluções Sênior</t>
         </is>
       </c>
-      <c r="B5" s="19" t="inlineStr">
+      <c r="B5" s="18" t="inlineStr">
         <is>
           <t>Brintell</t>
         </is>
       </c>
-      <c r="C5" s="17">
+      <c r="C5" s="16">
         <f>Papéis!D5</f>
         <v/>
       </c>
-      <c r="D5" s="20">
+      <c r="D5" s="19">
         <f>SUMPRODUCT(('Custo Detalhado'!$B$4:$B$200=A5)*'Custo Detalhado'!$D$4:$D$200*'Custo Detalhado'!$E$4:$E$200)</f>
         <v/>
       </c>
@@ -3834,7 +3875,7 @@
         <f>SUMIF('Custo Detalhado'!B:B,A5,'Custo Detalhado'!G:G)</f>
         <v/>
       </c>
-      <c r="F5" s="21">
+      <c r="F5" s="20">
         <f>E5/E14</f>
         <v/>
       </c>
@@ -3845,16 +3886,16 @@
           <t>Engenheiro de Dados Sênior — Pipelines/Tensores</t>
         </is>
       </c>
-      <c r="B6" s="19" t="inlineStr">
+      <c r="B6" s="18" t="inlineStr">
         <is>
           <t>Brintell</t>
         </is>
       </c>
-      <c r="C6" s="17">
+      <c r="C6" s="16">
         <f>Papéis!D6</f>
         <v/>
       </c>
-      <c r="D6" s="20">
+      <c r="D6" s="19">
         <f>SUMPRODUCT(('Custo Detalhado'!$B$4:$B$200=A6)*'Custo Detalhado'!$D$4:$D$200*'Custo Detalhado'!$E$4:$E$200)</f>
         <v/>
       </c>
@@ -3862,7 +3903,7 @@
         <f>SUMIF('Custo Detalhado'!B:B,A6,'Custo Detalhado'!G:G)</f>
         <v/>
       </c>
-      <c r="F6" s="21">
+      <c r="F6" s="20">
         <f>E6/E14</f>
         <v/>
       </c>
@@ -3873,16 +3914,16 @@
           <t>Cientista de Dados Sênior — ML/Personas/Markov/Bayes</t>
         </is>
       </c>
-      <c r="B7" s="19" t="inlineStr">
+      <c r="B7" s="18" t="inlineStr">
         <is>
           <t>Brintell</t>
         </is>
       </c>
-      <c r="C7" s="17">
+      <c r="C7" s="16">
         <f>Papéis!D7</f>
         <v/>
       </c>
-      <c r="D7" s="20">
+      <c r="D7" s="19">
         <f>SUMPRODUCT(('Custo Detalhado'!$B$4:$B$200=A7)*'Custo Detalhado'!$D$4:$D$200*'Custo Detalhado'!$E$4:$E$200)</f>
         <v/>
       </c>
@@ -3890,7 +3931,7 @@
         <f>SUMIF('Custo Detalhado'!B:B,A7,'Custo Detalhado'!G:G)</f>
         <v/>
       </c>
-      <c r="F7" s="21">
+      <c r="F7" s="20">
         <f>E7/E14</f>
         <v/>
       </c>
@@ -3901,16 +3942,16 @@
           <t>Engenheiro de Software Sênior — Dashboards/API</t>
         </is>
       </c>
-      <c r="B8" s="19" t="inlineStr">
+      <c r="B8" s="18" t="inlineStr">
         <is>
           <t>Brintell</t>
         </is>
       </c>
-      <c r="C8" s="17">
+      <c r="C8" s="16">
         <f>Papéis!D8</f>
         <v/>
       </c>
-      <c r="D8" s="20">
+      <c r="D8" s="19">
         <f>SUMPRODUCT(('Custo Detalhado'!$B$4:$B$200=A8)*'Custo Detalhado'!$D$4:$D$200*'Custo Detalhado'!$E$4:$E$200)</f>
         <v/>
       </c>
@@ -3918,7 +3959,7 @@
         <f>SUMIF('Custo Detalhado'!B:B,A8,'Custo Detalhado'!G:G)</f>
         <v/>
       </c>
-      <c r="F8" s="21">
+      <c r="F8" s="20">
         <f>E8/E14</f>
         <v/>
       </c>
@@ -3929,16 +3970,16 @@
           <t>Engenheiro de Dados Sênior — MLOps/Streaming</t>
         </is>
       </c>
-      <c r="B9" s="19" t="inlineStr">
+      <c r="B9" s="18" t="inlineStr">
         <is>
           <t>Brintell</t>
         </is>
       </c>
-      <c r="C9" s="17">
+      <c r="C9" s="16">
         <f>Papéis!D9</f>
         <v/>
       </c>
-      <c r="D9" s="20">
+      <c r="D9" s="19">
         <f>SUMPRODUCT(('Custo Detalhado'!$B$4:$B$200=A9)*'Custo Detalhado'!$D$4:$D$200*'Custo Detalhado'!$E$4:$E$200)</f>
         <v/>
       </c>
@@ -3946,7 +3987,7 @@
         <f>SUMIF('Custo Detalhado'!B:B,A9,'Custo Detalhado'!G:G)</f>
         <v/>
       </c>
-      <c r="F9" s="21">
+      <c r="F9" s="20">
         <f>E9/E14</f>
         <v/>
       </c>
@@ -3957,16 +3998,16 @@
           <t>Rafael — Eng. CDRVIEW Sênior (Parser/Ingestão/Redução/API)</t>
         </is>
       </c>
-      <c r="B10" s="16" t="inlineStr">
+      <c r="B10" s="15" t="inlineStr">
         <is>
           <t>Claro/CDRVIEW</t>
         </is>
       </c>
-      <c r="C10" s="17">
+      <c r="C10" s="16">
         <f>Papéis!D10</f>
         <v/>
       </c>
-      <c r="D10" s="20">
+      <c r="D10" s="19">
         <f>SUMPRODUCT(('Custo Detalhado'!$B$4:$B$200=A10)*'Custo Detalhado'!$D$4:$D$200*'Custo Detalhado'!$E$4:$E$200)</f>
         <v/>
       </c>
@@ -3974,7 +4015,7 @@
         <f>SUMIF('Custo Detalhado'!B:B,A10,'Custo Detalhado'!G:G)</f>
         <v/>
       </c>
-      <c r="F10" s="21">
+      <c r="F10" s="20">
         <f>E10/E14</f>
         <v/>
       </c>
@@ -3985,16 +4026,16 @@
           <t>Feijão — Eng. CDRVIEW Sênior (Alarmística online/API)</t>
         </is>
       </c>
-      <c r="B11" s="16" t="inlineStr">
+      <c r="B11" s="15" t="inlineStr">
         <is>
           <t>Claro/CDRVIEW</t>
         </is>
       </c>
-      <c r="C11" s="17">
+      <c r="C11" s="16">
         <f>Papéis!D11</f>
         <v/>
       </c>
-      <c r="D11" s="20">
+      <c r="D11" s="19">
         <f>SUMPRODUCT(('Custo Detalhado'!$B$4:$B$200=A11)*'Custo Detalhado'!$D$4:$D$200*'Custo Detalhado'!$E$4:$E$200)</f>
         <v/>
       </c>
@@ -4002,7 +4043,7 @@
         <f>SUMIF('Custo Detalhado'!B:B,A11,'Custo Detalhado'!G:G)</f>
         <v/>
       </c>
-      <c r="F11" s="21">
+      <c r="F11" s="20">
         <f>E11/E14</f>
         <v/>
       </c>
@@ -4013,16 +4054,16 @@
           <t>Andréia — QA Sênior</t>
         </is>
       </c>
-      <c r="B12" s="16" t="inlineStr">
+      <c r="B12" s="15" t="inlineStr">
         <is>
           <t>Claro/CDRVIEW</t>
         </is>
       </c>
-      <c r="C12" s="17">
+      <c r="C12" s="16">
         <f>Papéis!D12</f>
         <v/>
       </c>
-      <c r="D12" s="20">
+      <c r="D12" s="19">
         <f>SUMPRODUCT(('Custo Detalhado'!$B$4:$B$200=A12)*'Custo Detalhado'!$D$4:$D$200*'Custo Detalhado'!$E$4:$E$200)</f>
         <v/>
       </c>
@@ -4030,7 +4071,7 @@
         <f>SUMIF('Custo Detalhado'!B:B,A12,'Custo Detalhado'!G:G)</f>
         <v/>
       </c>
-      <c r="F12" s="21">
+      <c r="F12" s="20">
         <f>E12/E14</f>
         <v/>
       </c>
@@ -4041,16 +4082,16 @@
           <t>CS — Implantação/Rollout</t>
         </is>
       </c>
-      <c r="B13" s="16" t="inlineStr">
+      <c r="B13" s="15" t="inlineStr">
         <is>
           <t>Claro</t>
         </is>
       </c>
-      <c r="C13" s="17">
+      <c r="C13" s="16">
         <f>Papéis!D13</f>
         <v/>
       </c>
-      <c r="D13" s="20">
+      <c r="D13" s="19">
         <f>SUMPRODUCT(('Custo Detalhado'!$B$4:$B$200=A13)*'Custo Detalhado'!$D$4:$D$200*'Custo Detalhado'!$E$4:$E$200)</f>
         <v/>
       </c>
@@ -4058,25 +4099,25 @@
         <f>SUMIF('Custo Detalhado'!B:B,A13,'Custo Detalhado'!G:G)</f>
         <v/>
       </c>
-      <c r="F13" s="21">
+      <c r="F13" s="20">
         <f>E13/E14</f>
         <v/>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="12" t="inlineStr">
+      <c r="A14" s="11" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B14" s="12" t="n"/>
-      <c r="C14" s="12" t="n"/>
-      <c r="D14" s="12" t="n"/>
-      <c r="E14" s="13">
+      <c r="B14" s="11" t="n"/>
+      <c r="C14" s="11" t="n"/>
+      <c r="D14" s="11" t="n"/>
+      <c r="E14" s="12">
         <f>SUM(E4:E13)</f>
         <v/>
       </c>
-      <c r="F14" s="12" t="n"/>
+      <c r="F14" s="11" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>